<commit_message>
NMR: certified practitioners whose websites mention NMR (tag in directory, table on NMR page)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/downloads/doctors.xlsx
+++ b/downloads/doctors.xlsx
@@ -706,9 +706,9 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Bigelow, Brian T</t>
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>Bigelow, Brian T mentions NMR</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
@@ -760,9 +760,9 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>Bisaccia, John Jalso in: Other chiropractors (CV and website review)</t>
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>Bisaccia, John J mentions NMRalso in: Other chiropractors (CV and website review)</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
@@ -783,9 +783,9 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>Bisaccia, Marna Malso in: Other chiropractors (CV and website review)</t>
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>Bisaccia, Marna M mentions NMRalso in: Other chiropractors (CV and website review)</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
@@ -829,9 +829,9 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>Cayer, Jeremy</t>
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>Cayer, Jeremy mentions NMR</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
@@ -1051,9 +1051,9 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>Duckett, Staceyalso in: Other chiropractors (CV and website review)</t>
+      <c r="A25" s="3" t="inlineStr">
+        <is>
+          <t>Duckett, Stacey mentions NMRalso in: Other chiropractors (CV and website review)</t>
         </is>
       </c>
       <c r="B25" s="3" t="inlineStr">
@@ -1300,9 +1300,9 @@
       </c>
     </row>
     <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>Hallam, David</t>
+      <c r="A36" s="3" t="inlineStr">
+        <is>
+          <t>Hallam, David mentions NMR</t>
         </is>
       </c>
       <c r="B36" s="3" t="inlineStr">
@@ -1415,9 +1415,9 @@
       </c>
     </row>
     <row r="41">
-      <c r="A41" t="inlineStr">
-        <is>
-          <t>Johnson, Jeffrey</t>
+      <c r="A41" s="3" t="inlineStr">
+        <is>
+          <t>Johnson, Jeffrey mentions NMR</t>
         </is>
       </c>
       <c r="B41" s="3" t="inlineStr">
@@ -1837,9 +1837,9 @@
       </c>
     </row>
     <row r="59">
-      <c r="A59" t="inlineStr">
-        <is>
-          <t>Miller, Diane</t>
+      <c r="A59" s="3" t="inlineStr">
+        <is>
+          <t>Miller, Diane mentions NMR</t>
         </is>
       </c>
       <c r="B59" t="inlineStr"/>
@@ -1921,9 +1921,9 @@
       </c>
     </row>
     <row r="63">
-      <c r="A63" t="inlineStr">
-        <is>
-          <t>Mott, Lisa</t>
+      <c r="A63" s="3" t="inlineStr">
+        <is>
+          <t>Mott, Lisa mentions NMR</t>
         </is>
       </c>
       <c r="B63" s="3" t="inlineStr">
@@ -2012,9 +2012,9 @@
       <c r="E67" t="inlineStr"/>
     </row>
     <row r="68">
-      <c r="A68" t="inlineStr">
-        <is>
-          <t>Poane, Robert</t>
+      <c r="A68" s="3" t="inlineStr">
+        <is>
+          <t>Poane, Robert mentions NMR</t>
         </is>
       </c>
       <c r="B68" s="3" t="inlineStr">
@@ -2345,9 +2345,9 @@
       </c>
     </row>
     <row r="83">
-      <c r="A83" t="inlineStr">
-        <is>
-          <t>Townshend, Judith</t>
+      <c r="A83" s="3" t="inlineStr">
+        <is>
+          <t>Townshend, Judith mentions NMR</t>
         </is>
       </c>
       <c r="B83" s="3" t="inlineStr">
@@ -2647,9 +2647,9 @@
       <c r="E96" t="inlineStr"/>
     </row>
     <row r="97">
-      <c r="A97" t="inlineStr">
-        <is>
-          <t>Zollinger-Muench, Nicole</t>
+      <c r="A97" s="3" t="inlineStr">
+        <is>
+          <t>Zollinger-Muench, Nicole mentions NMR</t>
         </is>
       </c>
       <c r="B97" s="3" t="inlineStr">
@@ -15493,1671 +15493,1683 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B9" r:id="rId12"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C9" r:id="rId13"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E9" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B10" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C10" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D10" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E10" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B11" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C11" r:id="rId20"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D11" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E11" r:id="rId22"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B12" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C12" r:id="rId24"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E12" r:id="rId25"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B13" r:id="rId26"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C13" r:id="rId27"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E13" r:id="rId28"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B14" r:id="rId29"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C14" r:id="rId30"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E14" r:id="rId31"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B15" r:id="rId32"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C15" r:id="rId33"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D15" r:id="rId34"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E15" r:id="rId35"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B16" r:id="rId36"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C16" r:id="rId37"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E16" r:id="rId38"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B17" r:id="rId39"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C17" r:id="rId40"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E17" r:id="rId41"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B18" r:id="rId42"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C18" r:id="rId43"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D18" r:id="rId44"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E18" r:id="rId45"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B19" r:id="rId46"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C19" r:id="rId47"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D19" r:id="rId48"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E19" r:id="rId49"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C20" r:id="rId50"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E20" r:id="rId51"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D21" r:id="rId52"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C22" r:id="rId53"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E22" r:id="rId54"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B23" r:id="rId55"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D23" r:id="rId56"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E23" r:id="rId57"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B24" r:id="rId58"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E24" r:id="rId59"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B25" r:id="rId60"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C25" r:id="rId61"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D25" r:id="rId62"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E25" r:id="rId63"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B26" r:id="rId64"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C26" r:id="rId65"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D26" r:id="rId66"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E26" r:id="rId67"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C27" r:id="rId68"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D27" r:id="rId69"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E27" r:id="rId70"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B28" r:id="rId71"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D28" r:id="rId72"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E28" r:id="rId73"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D29" r:id="rId74"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C30" r:id="rId75"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D30" r:id="rId76"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E30" r:id="rId77"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B31" r:id="rId78"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C31" r:id="rId79"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E31" r:id="rId80"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D32" r:id="rId81"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B33" r:id="rId82"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D33" r:id="rId83"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E33" r:id="rId84"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B34" r:id="rId85"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C34" r:id="rId86"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D34" r:id="rId87"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E34" r:id="rId88"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C35" r:id="rId89"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D35" r:id="rId90"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E35" r:id="rId91"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B36" r:id="rId92"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C36" r:id="rId93"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E36" r:id="rId94"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B37" r:id="rId95"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C37" r:id="rId96"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D37" r:id="rId97"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E37" r:id="rId98"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B38" r:id="rId99"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C38" r:id="rId100"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E38" r:id="rId101"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C39" r:id="rId102"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E39" r:id="rId103"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C40" r:id="rId104"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D40" r:id="rId105"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E40" r:id="rId106"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B41" r:id="rId107"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D41" r:id="rId108"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E41" r:id="rId109"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B42" r:id="rId110"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C42" r:id="rId111"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D42" r:id="rId112"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E42" r:id="rId113"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C43" r:id="rId114"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D43" r:id="rId115"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E43" r:id="rId116"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C44" r:id="rId117"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D44" r:id="rId118"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E44" r:id="rId119"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B45" r:id="rId120"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D45" r:id="rId121"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E45" r:id="rId122"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D46" r:id="rId123"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B47" r:id="rId124"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C47" r:id="rId125"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D47" r:id="rId126"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E47" r:id="rId127"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C48" r:id="rId128"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D48" r:id="rId129"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E48" r:id="rId130"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B49" r:id="rId131"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E49" r:id="rId132"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B50" r:id="rId133"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C50" r:id="rId134"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D50" r:id="rId135"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E50" r:id="rId136"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B51" r:id="rId137"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C51" r:id="rId138"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D51" r:id="rId139"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E51" r:id="rId140"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B52" r:id="rId141"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D52" r:id="rId142"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E52" r:id="rId143"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B53" r:id="rId144"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D53" r:id="rId145"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E53" r:id="rId146"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C54" r:id="rId147"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D54" r:id="rId148"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E54" r:id="rId149"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B55" r:id="rId150"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C55" r:id="rId151"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E55" r:id="rId152"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C56" r:id="rId153"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D56" r:id="rId154"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E56" r:id="rId155"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C57" r:id="rId156"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D57" r:id="rId157"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E57" r:id="rId158"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B58" r:id="rId159"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C58" r:id="rId160"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D58" r:id="rId161"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E58" r:id="rId162"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C59" r:id="rId163"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E59" r:id="rId164"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D60" r:id="rId165"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B61" r:id="rId166"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C61" r:id="rId167"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D61" r:id="rId168"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E61" r:id="rId169"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B62" r:id="rId170"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C62" r:id="rId171"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E62" r:id="rId172"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B63" r:id="rId173"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C63" r:id="rId174"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E63" r:id="rId175"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B64" r:id="rId176"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E64" r:id="rId177"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B65" r:id="rId178"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D65" r:id="rId179"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E65" r:id="rId180"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D67" r:id="rId181"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B68" r:id="rId182"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C68" r:id="rId183"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D68" r:id="rId184"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E68" r:id="rId185"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D69" r:id="rId186"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C70" r:id="rId187"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D70" r:id="rId188"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E70" r:id="rId189"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B71" r:id="rId190"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E71" r:id="rId191"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C72" r:id="rId192"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E72" r:id="rId193"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B73" r:id="rId194"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D73" r:id="rId195"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E73" r:id="rId196"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B74" r:id="rId197"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C74" r:id="rId198"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D74" r:id="rId199"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E74" r:id="rId200"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B75" r:id="rId201"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C75" r:id="rId202"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D75" r:id="rId203"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E75" r:id="rId204"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B76" r:id="rId205"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C76" r:id="rId206"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E76" r:id="rId207"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B77" r:id="rId208"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C77" r:id="rId209"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D77" r:id="rId210"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E77" r:id="rId211"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B79" r:id="rId212"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D79" r:id="rId213"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E79" r:id="rId214"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B80" r:id="rId215"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C80" r:id="rId216"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E80" r:id="rId217"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B81" r:id="rId218"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C81" r:id="rId219"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D81" r:id="rId220"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E81" r:id="rId221"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C82" r:id="rId222"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E82" r:id="rId223"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B83" r:id="rId224"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C83" r:id="rId225"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D83" r:id="rId226"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E83" r:id="rId227"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B84" r:id="rId228"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C84" r:id="rId229"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D84" r:id="rId230"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E84" r:id="rId231"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B86" r:id="rId232"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C86" r:id="rId233"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E86" r:id="rId234"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C87" r:id="rId235"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E87" r:id="rId236"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B88" r:id="rId237"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C88" r:id="rId238"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E88" r:id="rId239"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C89" r:id="rId240"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D89" r:id="rId241"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E89" r:id="rId242"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C90" r:id="rId243"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D90" r:id="rId244"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E90" r:id="rId245"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B91" r:id="rId246"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C91" r:id="rId247"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E91" r:id="rId248"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B92" r:id="rId249"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C92" r:id="rId250"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E92" r:id="rId251"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B93" r:id="rId252"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C93" r:id="rId253"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E93" r:id="rId254"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C94" r:id="rId255"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D94" r:id="rId256"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E94" r:id="rId257"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B95" r:id="rId258"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D95" r:id="rId259"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E95" r:id="rId260"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B97" r:id="rId261"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C97" r:id="rId262"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E97" r:id="rId263"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B98" r:id="rId264"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C98" r:id="rId265"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E98" r:id="rId266"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D100" r:id="rId267"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D101" r:id="rId268"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D102" r:id="rId269"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B103" r:id="rId270"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D103" r:id="rId271"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E103" r:id="rId272"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D104" r:id="rId273"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D106" r:id="rId274"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D107" r:id="rId275"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D108" r:id="rId276"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D109" r:id="rId277"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D110" r:id="rId278"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C111" r:id="rId279"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E111" r:id="rId280"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D112" r:id="rId281"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D113" r:id="rId282"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B114" r:id="rId283"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E114" r:id="rId284"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D115" r:id="rId285"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D116" r:id="rId286"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D117" r:id="rId287"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D118" r:id="rId288"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D119" r:id="rId289"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B120" r:id="rId290"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E120" r:id="rId291"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D121" r:id="rId292"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D122" r:id="rId293"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D123" r:id="rId294"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D124" r:id="rId295"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D125" r:id="rId296"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D126" r:id="rId297"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D127" r:id="rId298"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D128" r:id="rId299"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D129" r:id="rId300"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B130" r:id="rId301"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C130" r:id="rId302"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D130" r:id="rId303"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E130" r:id="rId304"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B131" r:id="rId305"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E131" r:id="rId306"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D132" r:id="rId307"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D133" r:id="rId308"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D134" r:id="rId309"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D135" r:id="rId310"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C136" r:id="rId311"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D136" r:id="rId312"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E136" r:id="rId313"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D137" r:id="rId314"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D138" r:id="rId315"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D139" r:id="rId316"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B140" r:id="rId317"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E140" r:id="rId318"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D141" r:id="rId319"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D142" r:id="rId320"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D143" r:id="rId321"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B144" r:id="rId322"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C144" r:id="rId323"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E144" r:id="rId324"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D145" r:id="rId325"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D146" r:id="rId326"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D147" r:id="rId327"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C148" r:id="rId328"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E148" r:id="rId329"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B149" r:id="rId330"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D149" r:id="rId331"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E149" r:id="rId332"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D150" r:id="rId333"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D151" r:id="rId334"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D152" r:id="rId335"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D153" r:id="rId336"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D154" r:id="rId337"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D155" r:id="rId338"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D156" r:id="rId339"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D157" r:id="rId340"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D158" r:id="rId341"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D159" r:id="rId342"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B160" r:id="rId343"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E160" r:id="rId344"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D161" r:id="rId345"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D162" r:id="rId346"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D163" r:id="rId347"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D164" r:id="rId348"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D165" r:id="rId349"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D166" r:id="rId350"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D167" r:id="rId351"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D168" r:id="rId352"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D169" r:id="rId353"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D170" r:id="rId354"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D171" r:id="rId355"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D172" r:id="rId356"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D173" r:id="rId357"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C174" r:id="rId358"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E174" r:id="rId359"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D175" r:id="rId360"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D176" r:id="rId361"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D177" r:id="rId362"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D178" r:id="rId363"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D179" r:id="rId364"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D180" r:id="rId365"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D181" r:id="rId366"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D182" r:id="rId367"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D183" r:id="rId368"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D184" r:id="rId369"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B185" r:id="rId370"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E185" r:id="rId371"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C186" r:id="rId372"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E186" r:id="rId373"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D187" r:id="rId374"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D188" r:id="rId375"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D189" r:id="rId376"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B190" r:id="rId377"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C190" r:id="rId378"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D190" r:id="rId379"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E190" r:id="rId380"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B191" r:id="rId381"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D191" r:id="rId382"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E191" r:id="rId383"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D192" r:id="rId384"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D193" r:id="rId385"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B194" r:id="rId386"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E194" r:id="rId387"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D195" r:id="rId388"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C196" r:id="rId389"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E196" r:id="rId390"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D197" r:id="rId391"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D198" r:id="rId392"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D199" r:id="rId393"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D200" r:id="rId394"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D201" r:id="rId395"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D202" r:id="rId396"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D203" r:id="rId397"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B204" r:id="rId398"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E204" r:id="rId399"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D205" r:id="rId400"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D206" r:id="rId401"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D207" r:id="rId402"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D208" r:id="rId403"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B209" r:id="rId404"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E209" r:id="rId405"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B210" r:id="rId406"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E210" r:id="rId407"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D211" r:id="rId408"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D212" r:id="rId409"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D213" r:id="rId410"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D214" r:id="rId411"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D215" r:id="rId412"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D216" r:id="rId413"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D217" r:id="rId414"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D218" r:id="rId415"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C219" r:id="rId416"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D219" r:id="rId417"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E219" r:id="rId418"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D220" r:id="rId419"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D221" r:id="rId420"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D222" r:id="rId421"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D223" r:id="rId422"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D224" r:id="rId423"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D225" r:id="rId424"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D226" r:id="rId425"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D227" r:id="rId426"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D228" r:id="rId427"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B229" r:id="rId428"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D229" r:id="rId429"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E229" r:id="rId430"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B230" r:id="rId431"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D230" r:id="rId432"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E230" r:id="rId433"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D231" r:id="rId434"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D232" r:id="rId435"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B233" r:id="rId436"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D233" r:id="rId437"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E233" r:id="rId438"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B234" r:id="rId439"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E234" r:id="rId440"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D235" r:id="rId441"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B236" r:id="rId442"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E236" r:id="rId443"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D237" r:id="rId444"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B238" r:id="rId445"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D238" r:id="rId446"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E238" r:id="rId447"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D239" r:id="rId448"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D240" r:id="rId449"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D241" r:id="rId450"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D242" r:id="rId451"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D243" r:id="rId452"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D244" r:id="rId453"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D245" r:id="rId454"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B246" r:id="rId455"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E246" r:id="rId456"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C247" r:id="rId457"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D247" r:id="rId458"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E247" r:id="rId459"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D248" r:id="rId460"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D249" r:id="rId461"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D250" r:id="rId462"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D251" r:id="rId463"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B252" r:id="rId464"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D252" r:id="rId465"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E252" r:id="rId466"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D253" r:id="rId467"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D254" r:id="rId468"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D255" r:id="rId469"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B256" r:id="rId470"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D256" r:id="rId471"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E256" r:id="rId472"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D257" r:id="rId473"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D258" r:id="rId474"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D259" r:id="rId475"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D260" r:id="rId476"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D261" r:id="rId477"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D262" r:id="rId478"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D263" r:id="rId479"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B264" r:id="rId480"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E264" r:id="rId481"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D265" r:id="rId482"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D266" r:id="rId483"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D267" r:id="rId484"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D268" r:id="rId485"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D269" r:id="rId486"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D270" r:id="rId487"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D271" r:id="rId488"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D272" r:id="rId489"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D273" r:id="rId490"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D274" r:id="rId491"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D275" r:id="rId492"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D276" r:id="rId493"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D277" r:id="rId494"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D278" r:id="rId495"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D279" r:id="rId496"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D280" r:id="rId497"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B281" r:id="rId498"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E281" r:id="rId499"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B282" r:id="rId500"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C282" r:id="rId501"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D282" r:id="rId502"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E282" r:id="rId503"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D283" r:id="rId504"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D284" r:id="rId505"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D286" r:id="rId506"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D287" r:id="rId507"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D288" r:id="rId508"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D289" r:id="rId509"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B290" r:id="rId510"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C290" r:id="rId511"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D290" r:id="rId512"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E290" r:id="rId513"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B292" r:id="rId514"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E292" r:id="rId515"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B293" r:id="rId516"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C293" r:id="rId517"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E293" r:id="rId518"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B294" r:id="rId519"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C294" r:id="rId520"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E294" r:id="rId521"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B295" r:id="rId522"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E295" r:id="rId523"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B296" r:id="rId524"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C296" r:id="rId525"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E296" r:id="rId526"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B297" r:id="rId527"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C297" r:id="rId528"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E297" r:id="rId529"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B298" r:id="rId530"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C298" r:id="rId531"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E298" r:id="rId532"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B299" r:id="rId533"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C299" r:id="rId534"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E299" r:id="rId535"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B300" r:id="rId536"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E300" r:id="rId537"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B301" r:id="rId538"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C301" r:id="rId539"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E301" r:id="rId540"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B302" r:id="rId541"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C302" r:id="rId542"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E302" r:id="rId543"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B303" r:id="rId544"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E303" r:id="rId545"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B304" r:id="rId546"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C304" r:id="rId547"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E304" r:id="rId548"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B305" r:id="rId549"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C305" r:id="rId550"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E305" r:id="rId551"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B306" r:id="rId552"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E306" r:id="rId553"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B307" r:id="rId554"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C307" r:id="rId555"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E307" r:id="rId556"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B308" r:id="rId557"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C308" r:id="rId558"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E308" r:id="rId559"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B309" r:id="rId560"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C309" r:id="rId561"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E309" r:id="rId562"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B310" r:id="rId563"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C310" r:id="rId564"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E310" r:id="rId565"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B311" r:id="rId566"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C311" r:id="rId567"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E311" r:id="rId568"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B312" r:id="rId569"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C312" r:id="rId570"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E312" r:id="rId571"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B313" r:id="rId572"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E313" r:id="rId573"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B314" r:id="rId574"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C314" r:id="rId575"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E314" r:id="rId576"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B315" r:id="rId577"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C315" r:id="rId578"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E315" r:id="rId579"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B316" r:id="rId580"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C316" r:id="rId581"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E316" r:id="rId582"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B317" r:id="rId583"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C317" r:id="rId584"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E317" r:id="rId585"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B318" r:id="rId586"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E318" r:id="rId587"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B319" r:id="rId588"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C319" r:id="rId589"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E319" r:id="rId590"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B320" r:id="rId591"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C320" r:id="rId592"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E320" r:id="rId593"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C322" r:id="rId594"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E322" r:id="rId595"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B323" r:id="rId596"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C323" r:id="rId597"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E323" r:id="rId598"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B324" r:id="rId599"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C324" r:id="rId600"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E324" r:id="rId601"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B325" r:id="rId602"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C325" r:id="rId603"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E325" r:id="rId604"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B326" r:id="rId605"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C326" r:id="rId606"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E326" r:id="rId607"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C327" r:id="rId608"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E327" r:id="rId609"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B328" r:id="rId610"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C328" r:id="rId611"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E328" r:id="rId612"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B329" r:id="rId613"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C329" r:id="rId614"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E329" r:id="rId615"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B330" r:id="rId616"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C330" r:id="rId617"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E330" r:id="rId618"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B331" r:id="rId619"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C331" r:id="rId620"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E331" r:id="rId621"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C332" r:id="rId622"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E332" r:id="rId623"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B333" r:id="rId624"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C333" r:id="rId625"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E333" r:id="rId626"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B334" r:id="rId627"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C334" r:id="rId628"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E334" r:id="rId629"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B335" r:id="rId630"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C335" r:id="rId631"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E335" r:id="rId632"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B336" r:id="rId633"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C336" r:id="rId634"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E336" r:id="rId635"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B337" r:id="rId636"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C337" r:id="rId637"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E337" r:id="rId638"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B338" r:id="rId639"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C338" r:id="rId640"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E338" r:id="rId641"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C339" r:id="rId642"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E339" r:id="rId643"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B340" r:id="rId644"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C340" r:id="rId645"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E340" r:id="rId646"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B341" r:id="rId647"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C341" r:id="rId648"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E341" r:id="rId649"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B342" r:id="rId650"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C342" r:id="rId651"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E342" r:id="rId652"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B343" r:id="rId653"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C343" r:id="rId654"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E343" r:id="rId655"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B344" r:id="rId656"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C344" r:id="rId657"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E344" r:id="rId658"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B345" r:id="rId659"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C345" r:id="rId660"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E345" r:id="rId661"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B346" r:id="rId662"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C346" r:id="rId663"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E346" r:id="rId664"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B347" r:id="rId665"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C347" r:id="rId666"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E347" r:id="rId667"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B348" r:id="rId668"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C348" r:id="rId669"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E348" r:id="rId670"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B349" r:id="rId671"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C349" r:id="rId672"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E349" r:id="rId673"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B350" r:id="rId674"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C350" r:id="rId675"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E350" r:id="rId676"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B351" r:id="rId677"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C351" r:id="rId678"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E351" r:id="rId679"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B352" r:id="rId680"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C352" r:id="rId681"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E352" r:id="rId682"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B353" r:id="rId683"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C353" r:id="rId684"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E353" r:id="rId685"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B354" r:id="rId686"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C354" r:id="rId687"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E354" r:id="rId688"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B355" r:id="rId689"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C355" r:id="rId690"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E355" r:id="rId691"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B356" r:id="rId692"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C356" r:id="rId693"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E356" r:id="rId694"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B357" r:id="rId695"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C357" r:id="rId696"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E357" r:id="rId697"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B358" r:id="rId698"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E358" r:id="rId699"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B359" r:id="rId700"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C359" r:id="rId701"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E359" r:id="rId702"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B360" r:id="rId703"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C360" r:id="rId704"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E360" r:id="rId705"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B361" r:id="rId706"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C361" r:id="rId707"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E361" r:id="rId708"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B362" r:id="rId709"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C362" r:id="rId710"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E362" r:id="rId711"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B363" r:id="rId712"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C363" r:id="rId713"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E363" r:id="rId714"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B364" r:id="rId715"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C364" r:id="rId716"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E364" r:id="rId717"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B365" r:id="rId718"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E365" r:id="rId719"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C366" r:id="rId720"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E366" r:id="rId721"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B367" r:id="rId722"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C367" r:id="rId723"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E367" r:id="rId724"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B368" r:id="rId725"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E368" r:id="rId726"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B369" r:id="rId727"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E369" r:id="rId728"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B370" r:id="rId729"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C370" r:id="rId730"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E370" r:id="rId731"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B371" r:id="rId732"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E371" r:id="rId733"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B372" r:id="rId734"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C372" r:id="rId735"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E372" r:id="rId736"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B373" r:id="rId737"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C373" r:id="rId738"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E373" r:id="rId739"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B374" r:id="rId740"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C374" r:id="rId741"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E374" r:id="rId742"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B375" r:id="rId743"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C375" r:id="rId744"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E375" r:id="rId745"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B376" r:id="rId746"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C376" r:id="rId747"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E376" r:id="rId748"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B377" r:id="rId749"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C377" r:id="rId750"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E377" r:id="rId751"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B378" r:id="rId752"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E378" r:id="rId753"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B379" r:id="rId754"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C379" r:id="rId755"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E379" r:id="rId756"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B380" r:id="rId757"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C380" r:id="rId758"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E380" r:id="rId759"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B381" r:id="rId760"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C381" r:id="rId761"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E381" r:id="rId762"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B382" r:id="rId763"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C382" r:id="rId764"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E382" r:id="rId765"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B383" r:id="rId766"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C383" r:id="rId767"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E383" r:id="rId768"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B384" r:id="rId769"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C384" r:id="rId770"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E384" r:id="rId771"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B385" r:id="rId772"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C385" r:id="rId773"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E385" r:id="rId774"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B386" r:id="rId775"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C386" r:id="rId776"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E386" r:id="rId777"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B387" r:id="rId778"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C387" r:id="rId779"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E387" r:id="rId780"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B388" r:id="rId781"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C388" r:id="rId782"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E388" r:id="rId783"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B389" r:id="rId784"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E389" r:id="rId785"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B390" r:id="rId786"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C390" r:id="rId787"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E390" r:id="rId788"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B391" r:id="rId789"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C391" r:id="rId790"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E391" r:id="rId791"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B392" r:id="rId792"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C392" r:id="rId793"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E392" r:id="rId794"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B393" r:id="rId795"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C393" r:id="rId796"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E393" r:id="rId797"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B394" r:id="rId798"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C394" r:id="rId799"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E394" r:id="rId800"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B395" r:id="rId801"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E395" r:id="rId802"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B396" r:id="rId803"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C396" r:id="rId804"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E396" r:id="rId805"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B397" r:id="rId806"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C397" r:id="rId807"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E397" r:id="rId808"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B398" r:id="rId809"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E398" r:id="rId810"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B399" r:id="rId811"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C399" r:id="rId812"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E399" r:id="rId813"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B400" r:id="rId814"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C400" r:id="rId815"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E400" r:id="rId816"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B401" r:id="rId817"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C401" r:id="rId818"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E401" r:id="rId819"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B402" r:id="rId820"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C402" r:id="rId821"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E402" r:id="rId822"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B403" r:id="rId823"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C403" r:id="rId824"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E403" r:id="rId825"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B404" r:id="rId826"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C404" r:id="rId827"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E404" r:id="rId828"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B405" r:id="rId829"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C405" r:id="rId830"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E405" r:id="rId831"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B406" r:id="rId832"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C406" r:id="rId833"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E406" r:id="rId834"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B407" r:id="rId835"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C407" r:id="rId836"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E407" r:id="rId837"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B408" r:id="rId838"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C408" r:id="rId839"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E408" r:id="rId840"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B409" r:id="rId841"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C409" r:id="rId842"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E409" r:id="rId843"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B410" r:id="rId844"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C410" r:id="rId845"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E410" r:id="rId846"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B411" r:id="rId847"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C411" r:id="rId848"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E411" r:id="rId849"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B412" r:id="rId850"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C412" r:id="rId851"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E412" r:id="rId852"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B413" r:id="rId853"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C413" r:id="rId854"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E413" r:id="rId855"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B414" r:id="rId856"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C414" r:id="rId857"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E414" r:id="rId858"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B415" r:id="rId859"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E415" r:id="rId860"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B416" r:id="rId861"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C416" r:id="rId862"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E416" r:id="rId863"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B417" r:id="rId864"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C417" r:id="rId865"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E417" r:id="rId866"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B418" r:id="rId867"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C418" r:id="rId868"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E418" r:id="rId869"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B419" r:id="rId870"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C419" r:id="rId871"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E419" r:id="rId872"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B420" r:id="rId873"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C420" r:id="rId874"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E420" r:id="rId875"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B421" r:id="rId876"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C421" r:id="rId877"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E421" r:id="rId878"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B422" r:id="rId879"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C422" r:id="rId880"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E422" r:id="rId881"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B423" r:id="rId882"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E423" r:id="rId883"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B424" r:id="rId884"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E424" r:id="rId885"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B425" r:id="rId886"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C425" r:id="rId887"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E425" r:id="rId888"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B426" r:id="rId889"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C426" r:id="rId890"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E426" r:id="rId891"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B427" r:id="rId892"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C427" r:id="rId893"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E427" r:id="rId894"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B428" r:id="rId895"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C428" r:id="rId896"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E428" r:id="rId897"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B429" r:id="rId898"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E429" r:id="rId899"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B430" r:id="rId900"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C430" r:id="rId901"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E430" r:id="rId902"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B431" r:id="rId903"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C431" r:id="rId904"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E431" r:id="rId905"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B432" r:id="rId906"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C432" r:id="rId907"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E432" r:id="rId908"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B433" r:id="rId909"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E433" r:id="rId910"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B434" r:id="rId911"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E434" r:id="rId912"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B435" r:id="rId913"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C435" r:id="rId914"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E435" r:id="rId915"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B436" r:id="rId916"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C436" r:id="rId917"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E436" r:id="rId918"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B437" r:id="rId919"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C437" r:id="rId920"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E437" r:id="rId921"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B438" r:id="rId922"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E438" r:id="rId923"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B439" r:id="rId924"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C439" r:id="rId925"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E439" r:id="rId926"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B440" r:id="rId927"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C440" r:id="rId928"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E440" r:id="rId929"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B441" r:id="rId930"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E441" r:id="rId931"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B442" r:id="rId932"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C442" r:id="rId933"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E442" r:id="rId934"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B443" r:id="rId935"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C443" r:id="rId936"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E443" r:id="rId937"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B444" r:id="rId938"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C444" r:id="rId939"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E444" r:id="rId940"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B445" r:id="rId941"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C445" r:id="rId942"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E445" r:id="rId943"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B446" r:id="rId944"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C446" r:id="rId945"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E446" r:id="rId946"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B447" r:id="rId947"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C447" r:id="rId948"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E447" r:id="rId949"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B448" r:id="rId950"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C448" r:id="rId951"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E448" r:id="rId952"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B449" r:id="rId953"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C449" r:id="rId954"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E449" r:id="rId955"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B450" r:id="rId956"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C450" r:id="rId957"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E450" r:id="rId958"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B451" r:id="rId959"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C451" r:id="rId960"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E451" r:id="rId961"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B452" r:id="rId962"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C452" r:id="rId963"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E452" r:id="rId964"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B453" r:id="rId965"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C453" r:id="rId966"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E453" r:id="rId967"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B454" r:id="rId968"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C454" r:id="rId969"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E454" r:id="rId970"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B455" r:id="rId971"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E455" r:id="rId972"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B456" r:id="rId973"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E456" r:id="rId974"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B457" r:id="rId975"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C457" r:id="rId976"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E457" r:id="rId977"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B458" r:id="rId978"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C458" r:id="rId979"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E458" r:id="rId980"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B459" r:id="rId981"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C459" r:id="rId982"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E459" r:id="rId983"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B460" r:id="rId984"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C460" r:id="rId985"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E460" r:id="rId986"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B461" r:id="rId987"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C461" r:id="rId988"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E461" r:id="rId989"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B462" r:id="rId990"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C462" r:id="rId991"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E462" r:id="rId992"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B463" r:id="rId993"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E463" r:id="rId994"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B464" r:id="rId995"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C464" r:id="rId996"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E464" r:id="rId997"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B465" r:id="rId998"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C465" r:id="rId999"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E465" r:id="rId1000"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B466" r:id="rId1001"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C466" r:id="rId1002"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E466" r:id="rId1003"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B467" r:id="rId1004"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C467" r:id="rId1005"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E467" r:id="rId1006"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C468" r:id="rId1007"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E468" r:id="rId1008"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B469" r:id="rId1009"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C469" r:id="rId1010"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E469" r:id="rId1011"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B470" r:id="rId1012"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C470" r:id="rId1013"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E470" r:id="rId1014"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B471" r:id="rId1015"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C471" r:id="rId1016"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E471" r:id="rId1017"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B472" r:id="rId1018"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C472" r:id="rId1019"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E472" r:id="rId1020"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B473" r:id="rId1021"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C473" r:id="rId1022"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E473" r:id="rId1023"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B474" r:id="rId1024"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C474" r:id="rId1025"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E474" r:id="rId1026"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B475" r:id="rId1027"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E475" r:id="rId1028"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B476" r:id="rId1029"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E476" r:id="rId1030"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B477" r:id="rId1031"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C477" r:id="rId1032"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E477" r:id="rId1033"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B478" r:id="rId1034"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E478" r:id="rId1035"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B479" r:id="rId1036"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E479" r:id="rId1037"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B480" r:id="rId1038"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C480" r:id="rId1039"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E480" r:id="rId1040"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B481" r:id="rId1041"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E481" r:id="rId1042"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B482" r:id="rId1043"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C482" r:id="rId1044"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E482" r:id="rId1045"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B483" r:id="rId1046"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C483" r:id="rId1047"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E483" r:id="rId1048"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C484" r:id="rId1049"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E484" r:id="rId1050"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B485" r:id="rId1051"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C485" r:id="rId1052"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E485" r:id="rId1053"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B486" r:id="rId1054"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C486" r:id="rId1055"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E486" r:id="rId1056"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B487" r:id="rId1057"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C487" r:id="rId1058"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E487" r:id="rId1059"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C488" r:id="rId1060"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E488" r:id="rId1061"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B489" r:id="rId1062"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C489" r:id="rId1063"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E489" r:id="rId1064"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B490" r:id="rId1065"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C490" r:id="rId1066"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E490" r:id="rId1067"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B491" r:id="rId1068"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C491" r:id="rId1069"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E491" r:id="rId1070"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B492" r:id="rId1071"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C492" r:id="rId1072"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E492" r:id="rId1073"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B493" r:id="rId1074"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C493" r:id="rId1075"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E493" r:id="rId1076"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B494" r:id="rId1077"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C494" r:id="rId1078"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E494" r:id="rId1079"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B495" r:id="rId1080"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C495" r:id="rId1081"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E495" r:id="rId1082"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B496" r:id="rId1083"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C496" r:id="rId1084"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E496" r:id="rId1085"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B497" r:id="rId1086"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C497" r:id="rId1087"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E497" r:id="rId1088"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B498" r:id="rId1089"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C498" r:id="rId1090"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E498" r:id="rId1091"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B499" r:id="rId1092"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C499" r:id="rId1093"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E499" r:id="rId1094"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B500" r:id="rId1095"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C500" r:id="rId1096"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E500" r:id="rId1097"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B501" r:id="rId1098"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C501" r:id="rId1099"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E501" r:id="rId1100"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B502" r:id="rId1101"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E502" r:id="rId1102"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B503" r:id="rId1103"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C503" r:id="rId1104"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E503" r:id="rId1105"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B504" r:id="rId1106"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C504" r:id="rId1107"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E504" r:id="rId1108"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B505" r:id="rId1109"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C505" r:id="rId1110"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E505" r:id="rId1111"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B506" r:id="rId1112"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C506" r:id="rId1113"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E506" r:id="rId1114"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B507" r:id="rId1115"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E507" r:id="rId1116"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B508" r:id="rId1117"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C508" r:id="rId1118"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E508" r:id="rId1119"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B509" r:id="rId1120"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C509" r:id="rId1121"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E509" r:id="rId1122"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B510" r:id="rId1123"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C510" r:id="rId1124"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E510" r:id="rId1125"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B511" r:id="rId1126"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C511" r:id="rId1127"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E511" r:id="rId1128"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B512" r:id="rId1129"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C512" r:id="rId1130"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E512" r:id="rId1131"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B513" r:id="rId1132"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C513" r:id="rId1133"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E513" r:id="rId1134"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B514" r:id="rId1135"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C514" r:id="rId1136"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E514" r:id="rId1137"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B515" r:id="rId1138"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C515" r:id="rId1139"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E515" r:id="rId1140"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B516" r:id="rId1141"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C516" r:id="rId1142"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E516" r:id="rId1143"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C517" r:id="rId1144"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E517" r:id="rId1145"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B518" r:id="rId1146"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C518" r:id="rId1147"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E518" r:id="rId1148"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B519" r:id="rId1149"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C519" r:id="rId1150"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E519" r:id="rId1151"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B520" r:id="rId1152"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C520" r:id="rId1153"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E520" r:id="rId1154"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B521" r:id="rId1155"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E521" r:id="rId1156"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B522" r:id="rId1157"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C522" r:id="rId1158"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E522" r:id="rId1159"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B523" r:id="rId1160"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C523" r:id="rId1161"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E523" r:id="rId1162"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B524" r:id="rId1163"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E524" r:id="rId1164"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B525" r:id="rId1165"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C525" r:id="rId1166"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E525" r:id="rId1167"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B526" r:id="rId1168"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C526" r:id="rId1169"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E526" r:id="rId1170"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C527" r:id="rId1171"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E527" r:id="rId1172"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B528" r:id="rId1173"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C528" r:id="rId1174"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E528" r:id="rId1175"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B529" r:id="rId1176"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C529" r:id="rId1177"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E529" r:id="rId1178"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B530" r:id="rId1179"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E530" r:id="rId1180"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B531" r:id="rId1181"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C531" r:id="rId1182"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E531" r:id="rId1183"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B532" r:id="rId1184"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C532" r:id="rId1185"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E532" r:id="rId1186"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B533" r:id="rId1187"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C533" r:id="rId1188"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E533" r:id="rId1189"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B534" r:id="rId1190"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C534" r:id="rId1191"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E534" r:id="rId1192"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B535" r:id="rId1193"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C535" r:id="rId1194"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E535" r:id="rId1195"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B536" r:id="rId1196"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C536" r:id="rId1197"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E536" r:id="rId1198"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B537" r:id="rId1199"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C537" r:id="rId1200"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E537" r:id="rId1201"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C538" r:id="rId1202"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E538" r:id="rId1203"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B539" r:id="rId1204"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E539" r:id="rId1205"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B540" r:id="rId1206"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C540" r:id="rId1207"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E540" r:id="rId1208"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B541" r:id="rId1209"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C541" r:id="rId1210"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E541" r:id="rId1211"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B542" r:id="rId1212"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C542" r:id="rId1213"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E542" r:id="rId1214"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B543" r:id="rId1215"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C543" r:id="rId1216"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E543" r:id="rId1217"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B545" r:id="rId1218"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E545" r:id="rId1219"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B546" r:id="rId1220"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C546" r:id="rId1221"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E546" r:id="rId1222"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B547" r:id="rId1223"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C547" r:id="rId1224"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E547" r:id="rId1225"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B548" r:id="rId1226"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C548" r:id="rId1227"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E548" r:id="rId1228"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B549" r:id="rId1229"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C549" r:id="rId1230"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E549" r:id="rId1231"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B551" r:id="rId1232"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E551" r:id="rId1233"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B552" r:id="rId1234"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E552" r:id="rId1235"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B553" r:id="rId1236"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C553" r:id="rId1237"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E553" r:id="rId1238"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B555" r:id="rId1239"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C555" r:id="rId1240"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E555" r:id="rId1241"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B556" r:id="rId1242"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C556" r:id="rId1243"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E556" r:id="rId1244"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B558" r:id="rId1245"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C558" r:id="rId1246"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E558" r:id="rId1247"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B560" r:id="rId1248"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C560" r:id="rId1249"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E560" r:id="rId1250"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B563" r:id="rId1251"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C563" r:id="rId1252"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E563" r:id="rId1253"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B564" r:id="rId1254"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E564" r:id="rId1255"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B565" r:id="rId1256"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E565" r:id="rId1257"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B566" r:id="rId1258"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C566" r:id="rId1259"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E566" r:id="rId1260"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B567" r:id="rId1261"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C567" r:id="rId1262"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E567" r:id="rId1263"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B568" r:id="rId1264"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E568" r:id="rId1265"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C569" r:id="rId1266"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E569" r:id="rId1267"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B570" r:id="rId1268"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E570" r:id="rId1269"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B571" r:id="rId1270"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C571" r:id="rId1271"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E571" r:id="rId1272"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B573" r:id="rId1273"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C573" r:id="rId1274"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E573" r:id="rId1275"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C574" r:id="rId1276"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E574" r:id="rId1277"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B575" r:id="rId1278"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C575" r:id="rId1279"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E575" r:id="rId1280"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B576" r:id="rId1281"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C576" r:id="rId1282"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E576" r:id="rId1283"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B577" r:id="rId1284"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C577" r:id="rId1285"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E577" r:id="rId1286"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B578" r:id="rId1287"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C578" r:id="rId1288"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E578" r:id="rId1289"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B579" r:id="rId1290"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C579" r:id="rId1291"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E579" r:id="rId1292"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B580" r:id="rId1293"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C580" r:id="rId1294"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E580" r:id="rId1295"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B581" r:id="rId1296"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C581" r:id="rId1297"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E581" r:id="rId1298"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B583" r:id="rId1299"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E583" r:id="rId1300"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B584" r:id="rId1301"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C584" r:id="rId1302"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E584" r:id="rId1303"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B587" r:id="rId1304"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C587" r:id="rId1305"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E587" r:id="rId1306"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B590" r:id="rId1307"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C590" r:id="rId1308"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E590" r:id="rId1309"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B591" r:id="rId1310"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C591" r:id="rId1311"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E591" r:id="rId1312"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B592" r:id="rId1313"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C592" r:id="rId1314"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E592" r:id="rId1315"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B593" r:id="rId1316"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C593" r:id="rId1317"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E593" r:id="rId1318"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B595" r:id="rId1319"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C595" r:id="rId1320"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E595" r:id="rId1321"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B596" r:id="rId1322"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C596" r:id="rId1323"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E596" r:id="rId1324"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C599" r:id="rId1325"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E599" r:id="rId1326"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B600" r:id="rId1327"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C600" r:id="rId1328"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E600" r:id="rId1329"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C601" r:id="rId1330"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E601" r:id="rId1331"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B602" r:id="rId1332"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C602" r:id="rId1333"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E602" r:id="rId1334"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C603" r:id="rId1335"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E603" r:id="rId1336"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B604" r:id="rId1337"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C604" r:id="rId1338"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E604" r:id="rId1339"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B605" r:id="rId1340"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C605" r:id="rId1341"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E605" r:id="rId1342"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B606" r:id="rId1343"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C606" r:id="rId1344"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E606" r:id="rId1345"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B607" r:id="rId1346"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C607" r:id="rId1347"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E607" r:id="rId1348"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B608" r:id="rId1349"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C608" r:id="rId1350"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E608" r:id="rId1351"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B609" r:id="rId1352"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C609" r:id="rId1353"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E609" r:id="rId1354"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B610" r:id="rId1355"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E610" r:id="rId1356"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C611" r:id="rId1357"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E611" r:id="rId1358"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C612" r:id="rId1359"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E612" r:id="rId1360"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C613" r:id="rId1361"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E613" r:id="rId1362"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B614" r:id="rId1363"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C614" r:id="rId1364"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E614" r:id="rId1365"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B615" r:id="rId1366"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E615" r:id="rId1367"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B616" r:id="rId1368"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E616" r:id="rId1369"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C617" r:id="rId1370"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E617" r:id="rId1371"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B618" r:id="rId1372"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C618" r:id="rId1373"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E618" r:id="rId1374"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C619" r:id="rId1375"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E619" r:id="rId1376"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C620" r:id="rId1377"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E620" r:id="rId1378"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C621" r:id="rId1379"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E621" r:id="rId1380"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C622" r:id="rId1381"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E622" r:id="rId1382"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B623" r:id="rId1383"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C623" r:id="rId1384"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E623" r:id="rId1385"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B624" r:id="rId1386"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C624" r:id="rId1387"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E624" r:id="rId1388"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B625" r:id="rId1389"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C625" r:id="rId1390"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E625" r:id="rId1391"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C626" r:id="rId1392"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E626" r:id="rId1393"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B627" r:id="rId1394"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C627" r:id="rId1395"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E627" r:id="rId1396"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C628" r:id="rId1397"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E628" r:id="rId1398"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B629" r:id="rId1399"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E629" r:id="rId1400"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C630" r:id="rId1401"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E630" r:id="rId1402"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B631" r:id="rId1403"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E631" r:id="rId1404"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B632" r:id="rId1405"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C632" r:id="rId1406"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E632" r:id="rId1407"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C633" r:id="rId1408"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E633" r:id="rId1409"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C634" r:id="rId1410"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E634" r:id="rId1411"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C635" r:id="rId1412"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E635" r:id="rId1413"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C636" r:id="rId1414"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E636" r:id="rId1415"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B637" r:id="rId1416"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C637" r:id="rId1417"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E637" r:id="rId1418"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B638" r:id="rId1419"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C638" r:id="rId1420"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E638" r:id="rId1421"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B639" r:id="rId1422"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E639" r:id="rId1423"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B640" r:id="rId1424"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C640" r:id="rId1425"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E640" r:id="rId1426"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B641" r:id="rId1427"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C641" r:id="rId1428"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E641" r:id="rId1429"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B642" r:id="rId1430"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C642" r:id="rId1431"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E642" r:id="rId1432"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C643" r:id="rId1433"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E643" r:id="rId1434"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C644" r:id="rId1435"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E644" r:id="rId1436"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C645" r:id="rId1437"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E645" r:id="rId1438"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C646" r:id="rId1439"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E646" r:id="rId1440"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C647" r:id="rId1441"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E647" r:id="rId1442"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B648" r:id="rId1443"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E648" r:id="rId1444"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C649" r:id="rId1445"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E649" r:id="rId1446"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B650" r:id="rId1447"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C650" r:id="rId1448"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E650" r:id="rId1449"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B651" r:id="rId1450"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C651" r:id="rId1451"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E651" r:id="rId1452"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B652" r:id="rId1453"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C652" r:id="rId1454"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E652" r:id="rId1455"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C653" r:id="rId1456"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E653" r:id="rId1457"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B654" r:id="rId1458"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C654" r:id="rId1459"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E654" r:id="rId1460"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B655" r:id="rId1461"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E655" r:id="rId1462"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B656" r:id="rId1463"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C656" r:id="rId1464"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E656" r:id="rId1465"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C657" r:id="rId1466"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E657" r:id="rId1467"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B658" r:id="rId1468"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E658" r:id="rId1469"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C659" r:id="rId1470"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E659" r:id="rId1471"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B660" r:id="rId1472"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C660" r:id="rId1473"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E660" r:id="rId1474"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C661" r:id="rId1475"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E661" r:id="rId1476"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C662" r:id="rId1477"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E662" r:id="rId1478"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B663" r:id="rId1479"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E663" r:id="rId1480"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C664" r:id="rId1481"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E664" r:id="rId1482"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C665" r:id="rId1483"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E665" r:id="rId1484"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B666" r:id="rId1485"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E666" r:id="rId1486"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B667" r:id="rId1487"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E667" r:id="rId1488"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C669" r:id="rId1489"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E669" r:id="rId1490"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B670" r:id="rId1491"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C670" r:id="rId1492"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E670" r:id="rId1493"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B671" r:id="rId1494"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C671" r:id="rId1495"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E671" r:id="rId1496"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B672" r:id="rId1497"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C672" r:id="rId1498"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E672" r:id="rId1499"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B673" r:id="rId1500"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C673" r:id="rId1501"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E673" r:id="rId1502"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B674" r:id="rId1503"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C674" r:id="rId1504"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E674" r:id="rId1505"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B675" r:id="rId1506"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C675" r:id="rId1507"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E675" r:id="rId1508"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C676" r:id="rId1509"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E676" r:id="rId1510"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B677" r:id="rId1511"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C677" r:id="rId1512"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E677" r:id="rId1513"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B678" r:id="rId1514"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E678" r:id="rId1515"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C679" r:id="rId1516"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E679" r:id="rId1517"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C680" r:id="rId1518"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E680" r:id="rId1519"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C681" r:id="rId1520"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E681" r:id="rId1521"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C682" r:id="rId1522"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E682" r:id="rId1523"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C683" r:id="rId1524"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E683" r:id="rId1525"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C684" r:id="rId1526"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E684" r:id="rId1527"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C685" r:id="rId1528"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E685" r:id="rId1529"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C686" r:id="rId1530"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E686" r:id="rId1531"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C687" r:id="rId1532"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E687" r:id="rId1533"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B688" r:id="rId1534"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C688" r:id="rId1535"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E688" r:id="rId1536"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B689" r:id="rId1537"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C689" r:id="rId1538"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E689" r:id="rId1539"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B690" r:id="rId1540"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C690" r:id="rId1541"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E690" r:id="rId1542"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B691" r:id="rId1543"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C691" r:id="rId1544"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E691" r:id="rId1545"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B692" r:id="rId1546"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C692" r:id="rId1547"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E692" r:id="rId1548"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C693" r:id="rId1549"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E693" r:id="rId1550"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B694" r:id="rId1551"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C694" r:id="rId1552"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E694" r:id="rId1553"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B695" r:id="rId1554"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C695" r:id="rId1555"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E695" r:id="rId1556"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B696" r:id="rId1557"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E696" r:id="rId1558"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C697" r:id="rId1559"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E697" r:id="rId1560"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B698" r:id="rId1561"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E698" r:id="rId1562"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C699" r:id="rId1563"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E699" r:id="rId1564"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B700" r:id="rId1565"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E700" r:id="rId1566"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B701" r:id="rId1567"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E701" r:id="rId1568"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B702" r:id="rId1569"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C702" r:id="rId1570"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E702" r:id="rId1571"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B703" r:id="rId1572"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E703" r:id="rId1573"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C704" r:id="rId1574"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E704" r:id="rId1575"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B705" r:id="rId1576"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C705" r:id="rId1577"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E705" r:id="rId1578"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C706" r:id="rId1579"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E706" r:id="rId1580"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B707" r:id="rId1581"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C707" r:id="rId1582"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E707" r:id="rId1583"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B708" r:id="rId1584"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C708" r:id="rId1585"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E708" r:id="rId1586"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C709" r:id="rId1587"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E709" r:id="rId1588"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C710" r:id="rId1589"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E710" r:id="rId1590"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C711" r:id="rId1591"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E711" r:id="rId1592"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B712" r:id="rId1593"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E712" r:id="rId1594"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B713" r:id="rId1595"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C713" r:id="rId1596"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E713" r:id="rId1597"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C714" r:id="rId1598"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E714" r:id="rId1599"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B715" r:id="rId1600"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C715" r:id="rId1601"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E715" r:id="rId1602"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B716" r:id="rId1603"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C716" r:id="rId1604"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E716" r:id="rId1605"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B718" r:id="rId1606"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C718" r:id="rId1607"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E718" r:id="rId1608"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D720" r:id="rId1609"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B721" r:id="rId1610"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E721" r:id="rId1611"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B722" r:id="rId1612"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E722" r:id="rId1613"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B723" r:id="rId1614"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E723" r:id="rId1615"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B724" r:id="rId1616"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E724" r:id="rId1617"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B725" r:id="rId1618"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C725" r:id="rId1619"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E725" r:id="rId1620"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B726" r:id="rId1621"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C726" r:id="rId1622"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E726" r:id="rId1623"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C727" r:id="rId1624"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E727" r:id="rId1625"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B728" r:id="rId1626"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C728" r:id="rId1627"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E728" r:id="rId1628"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B729" r:id="rId1629"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C729" r:id="rId1630"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E729" r:id="rId1631"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C730" r:id="rId1632"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E730" r:id="rId1633"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C731" r:id="rId1634"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E731" r:id="rId1635"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B732" r:id="rId1636"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C732" r:id="rId1637"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E732" r:id="rId1638"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B733" r:id="rId1639"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E733" r:id="rId1640"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B734" r:id="rId1641"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E734" r:id="rId1642"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B735" r:id="rId1643"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E735" r:id="rId1644"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B736" r:id="rId1645"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C736" r:id="rId1646"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E736" r:id="rId1647"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B737" r:id="rId1648"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E737" r:id="rId1649"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C738" r:id="rId1650"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E738" r:id="rId1651"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C739" r:id="rId1652"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E739" r:id="rId1653"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B740" r:id="rId1654"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C740" r:id="rId1655"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E740" r:id="rId1656"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B741" r:id="rId1657"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C741" r:id="rId1658"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E741" r:id="rId1659"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C742" r:id="rId1660"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E742" r:id="rId1661"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B743" r:id="rId1662"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C743" r:id="rId1663"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E743" r:id="rId1664"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C744" r:id="rId1665"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E744" r:id="rId1666"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B745" r:id="rId1667"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E745" r:id="rId1668"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B746" r:id="rId1669"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C746" r:id="rId1670"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E746" r:id="rId1671"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B747" r:id="rId1672"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E747" r:id="rId1673"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B748" r:id="rId1674"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C748" r:id="rId1675"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E748" r:id="rId1676"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B749" r:id="rId1677"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C749" r:id="rId1678"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E749" r:id="rId1679"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A10" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B10" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C10" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D10" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E10" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B11" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C11" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D11" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E11" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A12" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B12" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C12" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E12" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A13" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B13" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C13" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E13" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B14" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C14" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E14" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A15" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B15" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C15" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D15" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E15" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B16" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C16" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E16" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B17" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C17" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E17" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B18" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C18" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D18" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E18" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B19" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C19" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D19" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E19" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C20" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E20" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D21" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C22" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E22" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B23" r:id="rId59"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D23" r:id="rId60"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E23" r:id="rId61"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B24" r:id="rId62"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E24" r:id="rId63"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A25" r:id="rId64"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B25" r:id="rId65"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C25" r:id="rId66"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D25" r:id="rId67"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E25" r:id="rId68"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B26" r:id="rId69"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C26" r:id="rId70"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D26" r:id="rId71"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E26" r:id="rId72"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C27" r:id="rId73"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D27" r:id="rId74"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E27" r:id="rId75"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B28" r:id="rId76"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D28" r:id="rId77"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E28" r:id="rId78"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D29" r:id="rId79"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C30" r:id="rId80"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D30" r:id="rId81"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E30" r:id="rId82"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B31" r:id="rId83"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C31" r:id="rId84"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E31" r:id="rId85"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D32" r:id="rId86"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B33" r:id="rId87"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D33" r:id="rId88"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E33" r:id="rId89"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B34" r:id="rId90"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C34" r:id="rId91"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D34" r:id="rId92"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E34" r:id="rId93"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C35" r:id="rId94"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D35" r:id="rId95"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E35" r:id="rId96"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A36" r:id="rId97"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B36" r:id="rId98"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C36" r:id="rId99"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E36" r:id="rId100"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B37" r:id="rId101"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C37" r:id="rId102"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D37" r:id="rId103"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E37" r:id="rId104"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B38" r:id="rId105"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C38" r:id="rId106"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E38" r:id="rId107"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C39" r:id="rId108"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E39" r:id="rId109"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C40" r:id="rId110"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D40" r:id="rId111"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E40" r:id="rId112"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A41" r:id="rId113"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B41" r:id="rId114"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D41" r:id="rId115"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E41" r:id="rId116"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B42" r:id="rId117"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C42" r:id="rId118"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D42" r:id="rId119"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E42" r:id="rId120"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C43" r:id="rId121"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D43" r:id="rId122"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E43" r:id="rId123"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C44" r:id="rId124"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D44" r:id="rId125"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E44" r:id="rId126"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B45" r:id="rId127"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D45" r:id="rId128"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E45" r:id="rId129"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D46" r:id="rId130"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B47" r:id="rId131"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C47" r:id="rId132"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D47" r:id="rId133"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E47" r:id="rId134"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C48" r:id="rId135"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D48" r:id="rId136"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E48" r:id="rId137"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B49" r:id="rId138"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E49" r:id="rId139"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B50" r:id="rId140"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C50" r:id="rId141"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D50" r:id="rId142"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E50" r:id="rId143"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B51" r:id="rId144"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C51" r:id="rId145"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D51" r:id="rId146"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E51" r:id="rId147"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B52" r:id="rId148"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D52" r:id="rId149"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E52" r:id="rId150"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B53" r:id="rId151"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D53" r:id="rId152"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E53" r:id="rId153"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C54" r:id="rId154"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D54" r:id="rId155"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E54" r:id="rId156"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B55" r:id="rId157"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C55" r:id="rId158"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E55" r:id="rId159"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C56" r:id="rId160"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D56" r:id="rId161"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E56" r:id="rId162"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C57" r:id="rId163"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D57" r:id="rId164"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E57" r:id="rId165"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B58" r:id="rId166"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C58" r:id="rId167"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D58" r:id="rId168"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E58" r:id="rId169"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A59" r:id="rId170"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C59" r:id="rId171"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E59" r:id="rId172"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D60" r:id="rId173"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B61" r:id="rId174"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C61" r:id="rId175"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D61" r:id="rId176"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E61" r:id="rId177"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B62" r:id="rId178"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C62" r:id="rId179"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E62" r:id="rId180"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A63" r:id="rId181"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B63" r:id="rId182"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C63" r:id="rId183"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E63" r:id="rId184"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B64" r:id="rId185"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E64" r:id="rId186"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B65" r:id="rId187"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D65" r:id="rId188"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E65" r:id="rId189"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D67" r:id="rId190"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A68" r:id="rId191"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B68" r:id="rId192"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C68" r:id="rId193"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D68" r:id="rId194"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E68" r:id="rId195"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D69" r:id="rId196"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C70" r:id="rId197"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D70" r:id="rId198"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E70" r:id="rId199"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B71" r:id="rId200"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E71" r:id="rId201"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C72" r:id="rId202"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E72" r:id="rId203"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B73" r:id="rId204"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D73" r:id="rId205"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E73" r:id="rId206"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B74" r:id="rId207"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C74" r:id="rId208"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D74" r:id="rId209"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E74" r:id="rId210"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B75" r:id="rId211"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C75" r:id="rId212"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D75" r:id="rId213"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E75" r:id="rId214"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B76" r:id="rId215"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C76" r:id="rId216"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E76" r:id="rId217"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B77" r:id="rId218"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C77" r:id="rId219"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D77" r:id="rId220"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E77" r:id="rId221"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B79" r:id="rId222"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D79" r:id="rId223"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E79" r:id="rId224"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B80" r:id="rId225"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C80" r:id="rId226"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E80" r:id="rId227"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B81" r:id="rId228"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C81" r:id="rId229"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D81" r:id="rId230"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E81" r:id="rId231"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C82" r:id="rId232"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E82" r:id="rId233"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A83" r:id="rId234"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B83" r:id="rId235"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C83" r:id="rId236"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D83" r:id="rId237"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E83" r:id="rId238"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B84" r:id="rId239"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C84" r:id="rId240"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D84" r:id="rId241"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E84" r:id="rId242"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B86" r:id="rId243"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C86" r:id="rId244"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E86" r:id="rId245"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C87" r:id="rId246"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E87" r:id="rId247"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B88" r:id="rId248"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C88" r:id="rId249"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E88" r:id="rId250"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C89" r:id="rId251"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D89" r:id="rId252"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E89" r:id="rId253"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C90" r:id="rId254"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D90" r:id="rId255"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E90" r:id="rId256"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B91" r:id="rId257"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C91" r:id="rId258"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E91" r:id="rId259"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B92" r:id="rId260"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C92" r:id="rId261"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E92" r:id="rId262"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B93" r:id="rId263"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C93" r:id="rId264"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E93" r:id="rId265"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C94" r:id="rId266"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D94" r:id="rId267"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E94" r:id="rId268"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B95" r:id="rId269"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D95" r:id="rId270"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E95" r:id="rId271"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A97" r:id="rId272"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B97" r:id="rId273"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C97" r:id="rId274"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E97" r:id="rId275"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B98" r:id="rId276"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C98" r:id="rId277"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E98" r:id="rId278"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D100" r:id="rId279"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D101" r:id="rId280"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D102" r:id="rId281"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B103" r:id="rId282"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D103" r:id="rId283"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E103" r:id="rId284"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D104" r:id="rId285"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D106" r:id="rId286"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D107" r:id="rId287"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D108" r:id="rId288"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D109" r:id="rId289"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D110" r:id="rId290"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C111" r:id="rId291"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E111" r:id="rId292"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D112" r:id="rId293"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D113" r:id="rId294"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B114" r:id="rId295"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E114" r:id="rId296"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D115" r:id="rId297"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D116" r:id="rId298"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D117" r:id="rId299"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D118" r:id="rId300"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D119" r:id="rId301"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B120" r:id="rId302"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E120" r:id="rId303"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D121" r:id="rId304"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D122" r:id="rId305"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D123" r:id="rId306"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D124" r:id="rId307"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D125" r:id="rId308"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D126" r:id="rId309"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D127" r:id="rId310"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D128" r:id="rId311"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D129" r:id="rId312"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B130" r:id="rId313"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C130" r:id="rId314"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D130" r:id="rId315"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E130" r:id="rId316"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B131" r:id="rId317"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E131" r:id="rId318"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D132" r:id="rId319"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D133" r:id="rId320"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D134" r:id="rId321"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D135" r:id="rId322"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C136" r:id="rId323"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D136" r:id="rId324"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E136" r:id="rId325"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D137" r:id="rId326"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D138" r:id="rId327"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D139" r:id="rId328"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B140" r:id="rId329"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E140" r:id="rId330"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D141" r:id="rId331"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D142" r:id="rId332"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D143" r:id="rId333"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B144" r:id="rId334"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C144" r:id="rId335"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E144" r:id="rId336"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D145" r:id="rId337"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D146" r:id="rId338"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D147" r:id="rId339"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C148" r:id="rId340"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E148" r:id="rId341"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B149" r:id="rId342"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D149" r:id="rId343"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E149" r:id="rId344"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D150" r:id="rId345"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D151" r:id="rId346"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D152" r:id="rId347"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D153" r:id="rId348"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D154" r:id="rId349"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D155" r:id="rId350"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D156" r:id="rId351"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D157" r:id="rId352"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D158" r:id="rId353"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D159" r:id="rId354"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B160" r:id="rId355"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E160" r:id="rId356"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D161" r:id="rId357"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D162" r:id="rId358"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D163" r:id="rId359"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D164" r:id="rId360"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D165" r:id="rId361"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D166" r:id="rId362"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D167" r:id="rId363"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D168" r:id="rId364"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D169" r:id="rId365"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D170" r:id="rId366"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D171" r:id="rId367"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D172" r:id="rId368"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D173" r:id="rId369"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C174" r:id="rId370"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E174" r:id="rId371"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D175" r:id="rId372"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D176" r:id="rId373"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D177" r:id="rId374"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D178" r:id="rId375"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D179" r:id="rId376"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D180" r:id="rId377"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D181" r:id="rId378"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D182" r:id="rId379"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D183" r:id="rId380"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D184" r:id="rId381"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B185" r:id="rId382"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E185" r:id="rId383"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C186" r:id="rId384"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E186" r:id="rId385"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D187" r:id="rId386"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D188" r:id="rId387"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D189" r:id="rId388"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B190" r:id="rId389"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C190" r:id="rId390"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D190" r:id="rId391"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E190" r:id="rId392"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B191" r:id="rId393"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D191" r:id="rId394"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E191" r:id="rId395"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D192" r:id="rId396"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D193" r:id="rId397"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B194" r:id="rId398"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E194" r:id="rId399"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D195" r:id="rId400"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C196" r:id="rId401"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E196" r:id="rId402"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D197" r:id="rId403"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D198" r:id="rId404"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D199" r:id="rId405"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D200" r:id="rId406"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D201" r:id="rId407"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D202" r:id="rId408"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D203" r:id="rId409"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B204" r:id="rId410"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E204" r:id="rId411"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D205" r:id="rId412"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D206" r:id="rId413"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D207" r:id="rId414"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D208" r:id="rId415"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B209" r:id="rId416"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E209" r:id="rId417"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B210" r:id="rId418"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E210" r:id="rId419"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D211" r:id="rId420"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D212" r:id="rId421"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D213" r:id="rId422"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D214" r:id="rId423"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D215" r:id="rId424"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D216" r:id="rId425"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D217" r:id="rId426"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D218" r:id="rId427"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C219" r:id="rId428"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D219" r:id="rId429"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E219" r:id="rId430"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D220" r:id="rId431"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D221" r:id="rId432"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D222" r:id="rId433"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D223" r:id="rId434"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D224" r:id="rId435"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D225" r:id="rId436"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D226" r:id="rId437"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D227" r:id="rId438"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D228" r:id="rId439"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B229" r:id="rId440"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D229" r:id="rId441"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E229" r:id="rId442"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B230" r:id="rId443"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D230" r:id="rId444"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E230" r:id="rId445"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D231" r:id="rId446"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D232" r:id="rId447"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B233" r:id="rId448"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D233" r:id="rId449"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E233" r:id="rId450"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B234" r:id="rId451"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E234" r:id="rId452"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D235" r:id="rId453"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B236" r:id="rId454"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E236" r:id="rId455"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D237" r:id="rId456"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B238" r:id="rId457"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D238" r:id="rId458"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E238" r:id="rId459"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D239" r:id="rId460"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D240" r:id="rId461"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D241" r:id="rId462"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D242" r:id="rId463"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D243" r:id="rId464"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D244" r:id="rId465"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D245" r:id="rId466"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B246" r:id="rId467"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E246" r:id="rId468"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C247" r:id="rId469"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D247" r:id="rId470"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E247" r:id="rId471"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D248" r:id="rId472"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D249" r:id="rId473"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D250" r:id="rId474"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D251" r:id="rId475"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B252" r:id="rId476"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D252" r:id="rId477"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E252" r:id="rId478"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D253" r:id="rId479"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D254" r:id="rId480"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D255" r:id="rId481"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B256" r:id="rId482"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D256" r:id="rId483"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E256" r:id="rId484"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D257" r:id="rId485"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D258" r:id="rId486"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D259" r:id="rId487"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D260" r:id="rId488"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D261" r:id="rId489"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D262" r:id="rId490"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D263" r:id="rId491"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B264" r:id="rId492"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E264" r:id="rId493"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D265" r:id="rId494"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D266" r:id="rId495"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D267" r:id="rId496"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D268" r:id="rId497"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D269" r:id="rId498"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D270" r:id="rId499"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D271" r:id="rId500"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D272" r:id="rId501"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D273" r:id="rId502"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D274" r:id="rId503"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D275" r:id="rId504"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D276" r:id="rId505"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D277" r:id="rId506"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D278" r:id="rId507"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D279" r:id="rId508"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D280" r:id="rId509"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B281" r:id="rId510"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E281" r:id="rId511"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B282" r:id="rId512"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C282" r:id="rId513"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D282" r:id="rId514"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E282" r:id="rId515"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D283" r:id="rId516"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D284" r:id="rId517"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D286" r:id="rId518"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D287" r:id="rId519"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D288" r:id="rId520"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D289" r:id="rId521"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B290" r:id="rId522"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C290" r:id="rId523"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D290" r:id="rId524"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E290" r:id="rId525"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B292" r:id="rId526"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E292" r:id="rId527"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B293" r:id="rId528"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C293" r:id="rId529"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E293" r:id="rId530"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B294" r:id="rId531"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C294" r:id="rId532"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E294" r:id="rId533"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B295" r:id="rId534"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E295" r:id="rId535"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B296" r:id="rId536"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C296" r:id="rId537"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E296" r:id="rId538"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B297" r:id="rId539"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C297" r:id="rId540"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E297" r:id="rId541"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B298" r:id="rId542"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C298" r:id="rId543"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E298" r:id="rId544"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B299" r:id="rId545"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C299" r:id="rId546"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E299" r:id="rId547"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B300" r:id="rId548"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E300" r:id="rId549"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B301" r:id="rId550"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C301" r:id="rId551"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E301" r:id="rId552"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B302" r:id="rId553"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C302" r:id="rId554"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E302" r:id="rId555"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B303" r:id="rId556"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E303" r:id="rId557"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B304" r:id="rId558"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C304" r:id="rId559"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E304" r:id="rId560"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B305" r:id="rId561"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C305" r:id="rId562"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E305" r:id="rId563"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B306" r:id="rId564"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E306" r:id="rId565"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B307" r:id="rId566"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C307" r:id="rId567"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E307" r:id="rId568"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B308" r:id="rId569"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C308" r:id="rId570"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E308" r:id="rId571"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B309" r:id="rId572"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C309" r:id="rId573"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E309" r:id="rId574"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B310" r:id="rId575"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C310" r:id="rId576"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E310" r:id="rId577"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B311" r:id="rId578"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C311" r:id="rId579"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E311" r:id="rId580"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B312" r:id="rId581"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C312" r:id="rId582"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E312" r:id="rId583"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B313" r:id="rId584"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E313" r:id="rId585"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B314" r:id="rId586"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C314" r:id="rId587"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E314" r:id="rId588"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B315" r:id="rId589"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C315" r:id="rId590"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E315" r:id="rId591"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B316" r:id="rId592"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C316" r:id="rId593"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E316" r:id="rId594"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B317" r:id="rId595"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C317" r:id="rId596"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E317" r:id="rId597"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B318" r:id="rId598"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E318" r:id="rId599"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B319" r:id="rId600"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C319" r:id="rId601"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E319" r:id="rId602"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B320" r:id="rId603"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C320" r:id="rId604"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E320" r:id="rId605"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C322" r:id="rId606"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E322" r:id="rId607"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B323" r:id="rId608"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C323" r:id="rId609"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E323" r:id="rId610"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B324" r:id="rId611"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C324" r:id="rId612"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E324" r:id="rId613"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B325" r:id="rId614"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C325" r:id="rId615"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E325" r:id="rId616"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B326" r:id="rId617"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C326" r:id="rId618"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E326" r:id="rId619"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C327" r:id="rId620"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E327" r:id="rId621"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B328" r:id="rId622"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C328" r:id="rId623"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E328" r:id="rId624"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B329" r:id="rId625"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C329" r:id="rId626"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E329" r:id="rId627"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B330" r:id="rId628"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C330" r:id="rId629"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E330" r:id="rId630"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B331" r:id="rId631"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C331" r:id="rId632"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E331" r:id="rId633"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C332" r:id="rId634"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E332" r:id="rId635"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B333" r:id="rId636"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C333" r:id="rId637"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E333" r:id="rId638"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B334" r:id="rId639"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C334" r:id="rId640"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E334" r:id="rId641"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B335" r:id="rId642"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C335" r:id="rId643"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E335" r:id="rId644"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B336" r:id="rId645"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C336" r:id="rId646"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E336" r:id="rId647"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B337" r:id="rId648"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C337" r:id="rId649"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E337" r:id="rId650"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B338" r:id="rId651"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C338" r:id="rId652"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E338" r:id="rId653"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C339" r:id="rId654"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E339" r:id="rId655"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B340" r:id="rId656"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C340" r:id="rId657"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E340" r:id="rId658"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B341" r:id="rId659"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C341" r:id="rId660"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E341" r:id="rId661"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B342" r:id="rId662"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C342" r:id="rId663"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E342" r:id="rId664"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B343" r:id="rId665"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C343" r:id="rId666"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E343" r:id="rId667"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B344" r:id="rId668"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C344" r:id="rId669"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E344" r:id="rId670"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B345" r:id="rId671"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C345" r:id="rId672"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E345" r:id="rId673"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B346" r:id="rId674"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C346" r:id="rId675"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E346" r:id="rId676"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B347" r:id="rId677"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C347" r:id="rId678"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E347" r:id="rId679"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B348" r:id="rId680"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C348" r:id="rId681"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E348" r:id="rId682"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B349" r:id="rId683"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C349" r:id="rId684"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E349" r:id="rId685"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B350" r:id="rId686"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C350" r:id="rId687"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E350" r:id="rId688"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B351" r:id="rId689"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C351" r:id="rId690"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E351" r:id="rId691"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B352" r:id="rId692"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C352" r:id="rId693"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E352" r:id="rId694"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B353" r:id="rId695"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C353" r:id="rId696"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E353" r:id="rId697"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B354" r:id="rId698"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C354" r:id="rId699"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E354" r:id="rId700"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B355" r:id="rId701"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C355" r:id="rId702"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E355" r:id="rId703"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B356" r:id="rId704"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C356" r:id="rId705"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E356" r:id="rId706"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B357" r:id="rId707"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C357" r:id="rId708"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E357" r:id="rId709"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B358" r:id="rId710"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E358" r:id="rId711"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B359" r:id="rId712"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C359" r:id="rId713"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E359" r:id="rId714"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B360" r:id="rId715"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C360" r:id="rId716"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E360" r:id="rId717"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B361" r:id="rId718"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C361" r:id="rId719"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E361" r:id="rId720"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B362" r:id="rId721"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C362" r:id="rId722"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E362" r:id="rId723"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B363" r:id="rId724"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C363" r:id="rId725"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E363" r:id="rId726"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B364" r:id="rId727"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C364" r:id="rId728"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E364" r:id="rId729"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B365" r:id="rId730"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E365" r:id="rId731"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C366" r:id="rId732"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E366" r:id="rId733"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B367" r:id="rId734"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C367" r:id="rId735"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E367" r:id="rId736"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B368" r:id="rId737"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E368" r:id="rId738"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B369" r:id="rId739"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E369" r:id="rId740"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B370" r:id="rId741"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C370" r:id="rId742"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E370" r:id="rId743"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B371" r:id="rId744"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E371" r:id="rId745"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B372" r:id="rId746"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C372" r:id="rId747"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E372" r:id="rId748"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B373" r:id="rId749"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C373" r:id="rId750"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E373" r:id="rId751"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B374" r:id="rId752"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C374" r:id="rId753"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E374" r:id="rId754"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B375" r:id="rId755"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C375" r:id="rId756"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E375" r:id="rId757"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B376" r:id="rId758"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C376" r:id="rId759"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E376" r:id="rId760"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B377" r:id="rId761"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C377" r:id="rId762"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E377" r:id="rId763"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B378" r:id="rId764"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E378" r:id="rId765"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B379" r:id="rId766"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C379" r:id="rId767"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E379" r:id="rId768"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B380" r:id="rId769"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C380" r:id="rId770"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E380" r:id="rId771"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B381" r:id="rId772"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C381" r:id="rId773"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E381" r:id="rId774"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B382" r:id="rId775"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C382" r:id="rId776"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E382" r:id="rId777"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B383" r:id="rId778"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C383" r:id="rId779"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E383" r:id="rId780"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B384" r:id="rId781"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C384" r:id="rId782"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E384" r:id="rId783"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B385" r:id="rId784"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C385" r:id="rId785"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E385" r:id="rId786"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B386" r:id="rId787"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C386" r:id="rId788"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E386" r:id="rId789"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B387" r:id="rId790"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C387" r:id="rId791"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E387" r:id="rId792"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B388" r:id="rId793"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C388" r:id="rId794"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E388" r:id="rId795"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B389" r:id="rId796"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E389" r:id="rId797"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B390" r:id="rId798"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C390" r:id="rId799"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E390" r:id="rId800"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B391" r:id="rId801"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C391" r:id="rId802"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E391" r:id="rId803"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B392" r:id="rId804"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C392" r:id="rId805"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E392" r:id="rId806"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B393" r:id="rId807"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C393" r:id="rId808"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E393" r:id="rId809"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B394" r:id="rId810"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C394" r:id="rId811"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E394" r:id="rId812"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B395" r:id="rId813"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E395" r:id="rId814"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B396" r:id="rId815"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C396" r:id="rId816"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E396" r:id="rId817"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B397" r:id="rId818"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C397" r:id="rId819"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E397" r:id="rId820"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B398" r:id="rId821"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E398" r:id="rId822"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B399" r:id="rId823"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C399" r:id="rId824"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E399" r:id="rId825"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B400" r:id="rId826"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C400" r:id="rId827"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E400" r:id="rId828"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B401" r:id="rId829"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C401" r:id="rId830"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E401" r:id="rId831"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B402" r:id="rId832"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C402" r:id="rId833"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E402" r:id="rId834"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B403" r:id="rId835"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C403" r:id="rId836"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E403" r:id="rId837"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B404" r:id="rId838"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C404" r:id="rId839"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E404" r:id="rId840"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B405" r:id="rId841"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C405" r:id="rId842"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E405" r:id="rId843"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B406" r:id="rId844"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C406" r:id="rId845"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E406" r:id="rId846"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B407" r:id="rId847"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C407" r:id="rId848"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E407" r:id="rId849"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B408" r:id="rId850"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C408" r:id="rId851"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E408" r:id="rId852"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B409" r:id="rId853"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C409" r:id="rId854"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E409" r:id="rId855"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B410" r:id="rId856"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C410" r:id="rId857"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E410" r:id="rId858"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B411" r:id="rId859"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C411" r:id="rId860"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E411" r:id="rId861"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B412" r:id="rId862"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C412" r:id="rId863"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E412" r:id="rId864"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B413" r:id="rId865"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C413" r:id="rId866"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E413" r:id="rId867"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B414" r:id="rId868"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C414" r:id="rId869"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E414" r:id="rId870"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B415" r:id="rId871"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E415" r:id="rId872"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B416" r:id="rId873"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C416" r:id="rId874"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E416" r:id="rId875"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B417" r:id="rId876"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C417" r:id="rId877"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E417" r:id="rId878"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B418" r:id="rId879"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C418" r:id="rId880"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E418" r:id="rId881"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B419" r:id="rId882"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C419" r:id="rId883"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E419" r:id="rId884"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B420" r:id="rId885"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C420" r:id="rId886"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E420" r:id="rId887"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B421" r:id="rId888"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C421" r:id="rId889"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E421" r:id="rId890"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B422" r:id="rId891"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C422" r:id="rId892"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E422" r:id="rId893"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B423" r:id="rId894"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E423" r:id="rId895"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B424" r:id="rId896"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E424" r:id="rId897"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B425" r:id="rId898"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C425" r:id="rId899"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E425" r:id="rId900"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B426" r:id="rId901"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C426" r:id="rId902"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E426" r:id="rId903"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B427" r:id="rId904"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C427" r:id="rId905"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E427" r:id="rId906"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B428" r:id="rId907"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C428" r:id="rId908"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E428" r:id="rId909"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B429" r:id="rId910"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E429" r:id="rId911"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B430" r:id="rId912"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C430" r:id="rId913"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E430" r:id="rId914"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B431" r:id="rId915"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C431" r:id="rId916"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E431" r:id="rId917"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B432" r:id="rId918"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C432" r:id="rId919"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E432" r:id="rId920"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B433" r:id="rId921"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E433" r:id="rId922"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B434" r:id="rId923"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E434" r:id="rId924"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B435" r:id="rId925"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C435" r:id="rId926"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E435" r:id="rId927"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B436" r:id="rId928"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C436" r:id="rId929"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E436" r:id="rId930"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B437" r:id="rId931"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C437" r:id="rId932"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E437" r:id="rId933"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B438" r:id="rId934"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E438" r:id="rId935"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B439" r:id="rId936"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C439" r:id="rId937"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E439" r:id="rId938"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B440" r:id="rId939"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C440" r:id="rId940"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E440" r:id="rId941"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B441" r:id="rId942"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E441" r:id="rId943"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B442" r:id="rId944"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C442" r:id="rId945"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E442" r:id="rId946"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B443" r:id="rId947"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C443" r:id="rId948"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E443" r:id="rId949"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B444" r:id="rId950"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C444" r:id="rId951"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E444" r:id="rId952"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B445" r:id="rId953"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C445" r:id="rId954"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E445" r:id="rId955"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B446" r:id="rId956"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C446" r:id="rId957"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E446" r:id="rId958"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B447" r:id="rId959"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C447" r:id="rId960"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E447" r:id="rId961"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B448" r:id="rId962"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C448" r:id="rId963"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E448" r:id="rId964"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B449" r:id="rId965"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C449" r:id="rId966"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E449" r:id="rId967"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B450" r:id="rId968"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C450" r:id="rId969"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E450" r:id="rId970"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B451" r:id="rId971"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C451" r:id="rId972"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E451" r:id="rId973"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B452" r:id="rId974"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C452" r:id="rId975"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E452" r:id="rId976"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B453" r:id="rId977"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C453" r:id="rId978"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E453" r:id="rId979"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B454" r:id="rId980"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C454" r:id="rId981"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E454" r:id="rId982"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B455" r:id="rId983"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E455" r:id="rId984"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B456" r:id="rId985"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E456" r:id="rId986"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B457" r:id="rId987"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C457" r:id="rId988"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E457" r:id="rId989"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B458" r:id="rId990"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C458" r:id="rId991"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E458" r:id="rId992"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B459" r:id="rId993"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C459" r:id="rId994"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E459" r:id="rId995"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B460" r:id="rId996"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C460" r:id="rId997"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E460" r:id="rId998"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B461" r:id="rId999"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C461" r:id="rId1000"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E461" r:id="rId1001"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B462" r:id="rId1002"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C462" r:id="rId1003"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E462" r:id="rId1004"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B463" r:id="rId1005"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E463" r:id="rId1006"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B464" r:id="rId1007"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C464" r:id="rId1008"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E464" r:id="rId1009"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B465" r:id="rId1010"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C465" r:id="rId1011"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E465" r:id="rId1012"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B466" r:id="rId1013"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C466" r:id="rId1014"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E466" r:id="rId1015"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B467" r:id="rId1016"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C467" r:id="rId1017"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E467" r:id="rId1018"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C468" r:id="rId1019"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E468" r:id="rId1020"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B469" r:id="rId1021"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C469" r:id="rId1022"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E469" r:id="rId1023"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B470" r:id="rId1024"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C470" r:id="rId1025"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E470" r:id="rId1026"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B471" r:id="rId1027"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C471" r:id="rId1028"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E471" r:id="rId1029"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B472" r:id="rId1030"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C472" r:id="rId1031"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E472" r:id="rId1032"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B473" r:id="rId1033"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C473" r:id="rId1034"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E473" r:id="rId1035"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B474" r:id="rId1036"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C474" r:id="rId1037"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E474" r:id="rId1038"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B475" r:id="rId1039"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E475" r:id="rId1040"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B476" r:id="rId1041"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E476" r:id="rId1042"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B477" r:id="rId1043"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C477" r:id="rId1044"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E477" r:id="rId1045"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B478" r:id="rId1046"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E478" r:id="rId1047"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B479" r:id="rId1048"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E479" r:id="rId1049"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B480" r:id="rId1050"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C480" r:id="rId1051"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E480" r:id="rId1052"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B481" r:id="rId1053"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E481" r:id="rId1054"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B482" r:id="rId1055"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C482" r:id="rId1056"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E482" r:id="rId1057"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B483" r:id="rId1058"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C483" r:id="rId1059"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E483" r:id="rId1060"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C484" r:id="rId1061"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E484" r:id="rId1062"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B485" r:id="rId1063"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C485" r:id="rId1064"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E485" r:id="rId1065"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B486" r:id="rId1066"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C486" r:id="rId1067"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E486" r:id="rId1068"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B487" r:id="rId1069"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C487" r:id="rId1070"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E487" r:id="rId1071"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C488" r:id="rId1072"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E488" r:id="rId1073"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B489" r:id="rId1074"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C489" r:id="rId1075"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E489" r:id="rId1076"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B490" r:id="rId1077"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C490" r:id="rId1078"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E490" r:id="rId1079"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B491" r:id="rId1080"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C491" r:id="rId1081"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E491" r:id="rId1082"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B492" r:id="rId1083"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C492" r:id="rId1084"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E492" r:id="rId1085"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B493" r:id="rId1086"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C493" r:id="rId1087"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E493" r:id="rId1088"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B494" r:id="rId1089"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C494" r:id="rId1090"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E494" r:id="rId1091"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B495" r:id="rId1092"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C495" r:id="rId1093"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E495" r:id="rId1094"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B496" r:id="rId1095"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C496" r:id="rId1096"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E496" r:id="rId1097"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B497" r:id="rId1098"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C497" r:id="rId1099"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E497" r:id="rId1100"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B498" r:id="rId1101"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C498" r:id="rId1102"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E498" r:id="rId1103"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B499" r:id="rId1104"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C499" r:id="rId1105"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E499" r:id="rId1106"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B500" r:id="rId1107"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C500" r:id="rId1108"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E500" r:id="rId1109"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B501" r:id="rId1110"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C501" r:id="rId1111"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E501" r:id="rId1112"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B502" r:id="rId1113"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E502" r:id="rId1114"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B503" r:id="rId1115"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C503" r:id="rId1116"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E503" r:id="rId1117"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B504" r:id="rId1118"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C504" r:id="rId1119"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E504" r:id="rId1120"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B505" r:id="rId1121"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C505" r:id="rId1122"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E505" r:id="rId1123"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B506" r:id="rId1124"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C506" r:id="rId1125"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E506" r:id="rId1126"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B507" r:id="rId1127"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E507" r:id="rId1128"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B508" r:id="rId1129"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C508" r:id="rId1130"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E508" r:id="rId1131"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B509" r:id="rId1132"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C509" r:id="rId1133"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E509" r:id="rId1134"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B510" r:id="rId1135"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C510" r:id="rId1136"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E510" r:id="rId1137"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B511" r:id="rId1138"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C511" r:id="rId1139"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E511" r:id="rId1140"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B512" r:id="rId1141"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C512" r:id="rId1142"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E512" r:id="rId1143"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B513" r:id="rId1144"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C513" r:id="rId1145"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E513" r:id="rId1146"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B514" r:id="rId1147"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C514" r:id="rId1148"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E514" r:id="rId1149"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B515" r:id="rId1150"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C515" r:id="rId1151"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E515" r:id="rId1152"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B516" r:id="rId1153"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C516" r:id="rId1154"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E516" r:id="rId1155"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C517" r:id="rId1156"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E517" r:id="rId1157"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B518" r:id="rId1158"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C518" r:id="rId1159"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E518" r:id="rId1160"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B519" r:id="rId1161"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C519" r:id="rId1162"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E519" r:id="rId1163"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B520" r:id="rId1164"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C520" r:id="rId1165"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E520" r:id="rId1166"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B521" r:id="rId1167"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E521" r:id="rId1168"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B522" r:id="rId1169"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C522" r:id="rId1170"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E522" r:id="rId1171"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B523" r:id="rId1172"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C523" r:id="rId1173"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E523" r:id="rId1174"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B524" r:id="rId1175"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E524" r:id="rId1176"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B525" r:id="rId1177"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C525" r:id="rId1178"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E525" r:id="rId1179"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B526" r:id="rId1180"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C526" r:id="rId1181"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E526" r:id="rId1182"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C527" r:id="rId1183"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E527" r:id="rId1184"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B528" r:id="rId1185"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C528" r:id="rId1186"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E528" r:id="rId1187"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B529" r:id="rId1188"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C529" r:id="rId1189"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E529" r:id="rId1190"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B530" r:id="rId1191"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E530" r:id="rId1192"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B531" r:id="rId1193"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C531" r:id="rId1194"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E531" r:id="rId1195"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B532" r:id="rId1196"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C532" r:id="rId1197"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E532" r:id="rId1198"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B533" r:id="rId1199"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C533" r:id="rId1200"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E533" r:id="rId1201"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B534" r:id="rId1202"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C534" r:id="rId1203"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E534" r:id="rId1204"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B535" r:id="rId1205"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C535" r:id="rId1206"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E535" r:id="rId1207"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B536" r:id="rId1208"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C536" r:id="rId1209"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E536" r:id="rId1210"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B537" r:id="rId1211"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C537" r:id="rId1212"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E537" r:id="rId1213"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C538" r:id="rId1214"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E538" r:id="rId1215"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B539" r:id="rId1216"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E539" r:id="rId1217"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B540" r:id="rId1218"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C540" r:id="rId1219"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E540" r:id="rId1220"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B541" r:id="rId1221"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C541" r:id="rId1222"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E541" r:id="rId1223"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B542" r:id="rId1224"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C542" r:id="rId1225"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E542" r:id="rId1226"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B543" r:id="rId1227"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C543" r:id="rId1228"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E543" r:id="rId1229"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B545" r:id="rId1230"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E545" r:id="rId1231"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B546" r:id="rId1232"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C546" r:id="rId1233"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E546" r:id="rId1234"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B547" r:id="rId1235"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C547" r:id="rId1236"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E547" r:id="rId1237"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B548" r:id="rId1238"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C548" r:id="rId1239"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E548" r:id="rId1240"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B549" r:id="rId1241"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C549" r:id="rId1242"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E549" r:id="rId1243"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B551" r:id="rId1244"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E551" r:id="rId1245"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B552" r:id="rId1246"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E552" r:id="rId1247"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B553" r:id="rId1248"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C553" r:id="rId1249"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E553" r:id="rId1250"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B555" r:id="rId1251"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C555" r:id="rId1252"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E555" r:id="rId1253"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B556" r:id="rId1254"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C556" r:id="rId1255"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E556" r:id="rId1256"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B558" r:id="rId1257"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C558" r:id="rId1258"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E558" r:id="rId1259"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B560" r:id="rId1260"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C560" r:id="rId1261"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E560" r:id="rId1262"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B563" r:id="rId1263"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C563" r:id="rId1264"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E563" r:id="rId1265"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B564" r:id="rId1266"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E564" r:id="rId1267"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B565" r:id="rId1268"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E565" r:id="rId1269"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B566" r:id="rId1270"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C566" r:id="rId1271"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E566" r:id="rId1272"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B567" r:id="rId1273"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C567" r:id="rId1274"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E567" r:id="rId1275"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B568" r:id="rId1276"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E568" r:id="rId1277"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C569" r:id="rId1278"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E569" r:id="rId1279"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B570" r:id="rId1280"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E570" r:id="rId1281"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B571" r:id="rId1282"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C571" r:id="rId1283"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E571" r:id="rId1284"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B573" r:id="rId1285"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C573" r:id="rId1286"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E573" r:id="rId1287"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C574" r:id="rId1288"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E574" r:id="rId1289"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B575" r:id="rId1290"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C575" r:id="rId1291"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E575" r:id="rId1292"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B576" r:id="rId1293"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C576" r:id="rId1294"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E576" r:id="rId1295"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B577" r:id="rId1296"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C577" r:id="rId1297"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E577" r:id="rId1298"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B578" r:id="rId1299"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C578" r:id="rId1300"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E578" r:id="rId1301"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B579" r:id="rId1302"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C579" r:id="rId1303"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E579" r:id="rId1304"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B580" r:id="rId1305"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C580" r:id="rId1306"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E580" r:id="rId1307"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B581" r:id="rId1308"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C581" r:id="rId1309"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E581" r:id="rId1310"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B583" r:id="rId1311"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E583" r:id="rId1312"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B584" r:id="rId1313"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C584" r:id="rId1314"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E584" r:id="rId1315"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B587" r:id="rId1316"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C587" r:id="rId1317"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E587" r:id="rId1318"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B590" r:id="rId1319"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C590" r:id="rId1320"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E590" r:id="rId1321"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B591" r:id="rId1322"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C591" r:id="rId1323"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E591" r:id="rId1324"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B592" r:id="rId1325"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C592" r:id="rId1326"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E592" r:id="rId1327"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B593" r:id="rId1328"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C593" r:id="rId1329"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E593" r:id="rId1330"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B595" r:id="rId1331"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C595" r:id="rId1332"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E595" r:id="rId1333"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B596" r:id="rId1334"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C596" r:id="rId1335"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E596" r:id="rId1336"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C599" r:id="rId1337"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E599" r:id="rId1338"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B600" r:id="rId1339"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C600" r:id="rId1340"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E600" r:id="rId1341"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C601" r:id="rId1342"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E601" r:id="rId1343"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B602" r:id="rId1344"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C602" r:id="rId1345"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E602" r:id="rId1346"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C603" r:id="rId1347"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E603" r:id="rId1348"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B604" r:id="rId1349"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C604" r:id="rId1350"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E604" r:id="rId1351"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B605" r:id="rId1352"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C605" r:id="rId1353"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E605" r:id="rId1354"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B606" r:id="rId1355"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C606" r:id="rId1356"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E606" r:id="rId1357"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B607" r:id="rId1358"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C607" r:id="rId1359"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E607" r:id="rId1360"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B608" r:id="rId1361"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C608" r:id="rId1362"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E608" r:id="rId1363"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B609" r:id="rId1364"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C609" r:id="rId1365"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E609" r:id="rId1366"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B610" r:id="rId1367"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E610" r:id="rId1368"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C611" r:id="rId1369"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E611" r:id="rId1370"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C612" r:id="rId1371"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E612" r:id="rId1372"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C613" r:id="rId1373"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E613" r:id="rId1374"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B614" r:id="rId1375"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C614" r:id="rId1376"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E614" r:id="rId1377"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B615" r:id="rId1378"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E615" r:id="rId1379"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B616" r:id="rId1380"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E616" r:id="rId1381"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C617" r:id="rId1382"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E617" r:id="rId1383"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B618" r:id="rId1384"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C618" r:id="rId1385"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E618" r:id="rId1386"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C619" r:id="rId1387"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E619" r:id="rId1388"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C620" r:id="rId1389"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E620" r:id="rId1390"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C621" r:id="rId1391"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E621" r:id="rId1392"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C622" r:id="rId1393"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E622" r:id="rId1394"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B623" r:id="rId1395"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C623" r:id="rId1396"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E623" r:id="rId1397"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B624" r:id="rId1398"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C624" r:id="rId1399"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E624" r:id="rId1400"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B625" r:id="rId1401"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C625" r:id="rId1402"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E625" r:id="rId1403"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C626" r:id="rId1404"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E626" r:id="rId1405"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B627" r:id="rId1406"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C627" r:id="rId1407"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E627" r:id="rId1408"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C628" r:id="rId1409"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E628" r:id="rId1410"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B629" r:id="rId1411"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E629" r:id="rId1412"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C630" r:id="rId1413"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E630" r:id="rId1414"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B631" r:id="rId1415"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E631" r:id="rId1416"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B632" r:id="rId1417"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C632" r:id="rId1418"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E632" r:id="rId1419"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C633" r:id="rId1420"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E633" r:id="rId1421"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C634" r:id="rId1422"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E634" r:id="rId1423"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C635" r:id="rId1424"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E635" r:id="rId1425"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C636" r:id="rId1426"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E636" r:id="rId1427"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B637" r:id="rId1428"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C637" r:id="rId1429"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E637" r:id="rId1430"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B638" r:id="rId1431"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C638" r:id="rId1432"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E638" r:id="rId1433"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B639" r:id="rId1434"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E639" r:id="rId1435"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B640" r:id="rId1436"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C640" r:id="rId1437"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E640" r:id="rId1438"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B641" r:id="rId1439"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C641" r:id="rId1440"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E641" r:id="rId1441"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B642" r:id="rId1442"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C642" r:id="rId1443"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E642" r:id="rId1444"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C643" r:id="rId1445"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E643" r:id="rId1446"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C644" r:id="rId1447"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E644" r:id="rId1448"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C645" r:id="rId1449"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E645" r:id="rId1450"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C646" r:id="rId1451"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E646" r:id="rId1452"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C647" r:id="rId1453"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E647" r:id="rId1454"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B648" r:id="rId1455"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E648" r:id="rId1456"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C649" r:id="rId1457"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E649" r:id="rId1458"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B650" r:id="rId1459"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C650" r:id="rId1460"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E650" r:id="rId1461"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B651" r:id="rId1462"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C651" r:id="rId1463"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E651" r:id="rId1464"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B652" r:id="rId1465"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C652" r:id="rId1466"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E652" r:id="rId1467"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C653" r:id="rId1468"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E653" r:id="rId1469"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B654" r:id="rId1470"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C654" r:id="rId1471"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E654" r:id="rId1472"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B655" r:id="rId1473"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E655" r:id="rId1474"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B656" r:id="rId1475"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C656" r:id="rId1476"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E656" r:id="rId1477"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C657" r:id="rId1478"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E657" r:id="rId1479"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B658" r:id="rId1480"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E658" r:id="rId1481"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C659" r:id="rId1482"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E659" r:id="rId1483"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B660" r:id="rId1484"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C660" r:id="rId1485"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E660" r:id="rId1486"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C661" r:id="rId1487"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E661" r:id="rId1488"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C662" r:id="rId1489"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E662" r:id="rId1490"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B663" r:id="rId1491"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E663" r:id="rId1492"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C664" r:id="rId1493"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E664" r:id="rId1494"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C665" r:id="rId1495"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E665" r:id="rId1496"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B666" r:id="rId1497"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E666" r:id="rId1498"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B667" r:id="rId1499"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E667" r:id="rId1500"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C669" r:id="rId1501"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E669" r:id="rId1502"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B670" r:id="rId1503"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C670" r:id="rId1504"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E670" r:id="rId1505"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B671" r:id="rId1506"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C671" r:id="rId1507"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E671" r:id="rId1508"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B672" r:id="rId1509"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C672" r:id="rId1510"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E672" r:id="rId1511"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B673" r:id="rId1512"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C673" r:id="rId1513"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E673" r:id="rId1514"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B674" r:id="rId1515"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C674" r:id="rId1516"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E674" r:id="rId1517"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B675" r:id="rId1518"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C675" r:id="rId1519"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E675" r:id="rId1520"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C676" r:id="rId1521"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E676" r:id="rId1522"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B677" r:id="rId1523"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C677" r:id="rId1524"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E677" r:id="rId1525"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B678" r:id="rId1526"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E678" r:id="rId1527"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C679" r:id="rId1528"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E679" r:id="rId1529"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C680" r:id="rId1530"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E680" r:id="rId1531"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C681" r:id="rId1532"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E681" r:id="rId1533"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C682" r:id="rId1534"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E682" r:id="rId1535"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C683" r:id="rId1536"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E683" r:id="rId1537"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C684" r:id="rId1538"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E684" r:id="rId1539"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C685" r:id="rId1540"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E685" r:id="rId1541"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C686" r:id="rId1542"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E686" r:id="rId1543"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C687" r:id="rId1544"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E687" r:id="rId1545"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B688" r:id="rId1546"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C688" r:id="rId1547"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E688" r:id="rId1548"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B689" r:id="rId1549"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C689" r:id="rId1550"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E689" r:id="rId1551"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B690" r:id="rId1552"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C690" r:id="rId1553"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E690" r:id="rId1554"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B691" r:id="rId1555"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C691" r:id="rId1556"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E691" r:id="rId1557"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B692" r:id="rId1558"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C692" r:id="rId1559"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E692" r:id="rId1560"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C693" r:id="rId1561"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E693" r:id="rId1562"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B694" r:id="rId1563"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C694" r:id="rId1564"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E694" r:id="rId1565"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B695" r:id="rId1566"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C695" r:id="rId1567"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E695" r:id="rId1568"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B696" r:id="rId1569"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E696" r:id="rId1570"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C697" r:id="rId1571"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E697" r:id="rId1572"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B698" r:id="rId1573"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E698" r:id="rId1574"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C699" r:id="rId1575"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E699" r:id="rId1576"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B700" r:id="rId1577"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E700" r:id="rId1578"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B701" r:id="rId1579"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E701" r:id="rId1580"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B702" r:id="rId1581"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C702" r:id="rId1582"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E702" r:id="rId1583"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B703" r:id="rId1584"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E703" r:id="rId1585"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C704" r:id="rId1586"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E704" r:id="rId1587"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B705" r:id="rId1588"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C705" r:id="rId1589"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E705" r:id="rId1590"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C706" r:id="rId1591"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E706" r:id="rId1592"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B707" r:id="rId1593"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C707" r:id="rId1594"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E707" r:id="rId1595"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B708" r:id="rId1596"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C708" r:id="rId1597"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E708" r:id="rId1598"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C709" r:id="rId1599"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E709" r:id="rId1600"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C710" r:id="rId1601"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E710" r:id="rId1602"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C711" r:id="rId1603"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E711" r:id="rId1604"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B712" r:id="rId1605"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E712" r:id="rId1606"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B713" r:id="rId1607"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C713" r:id="rId1608"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E713" r:id="rId1609"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C714" r:id="rId1610"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E714" r:id="rId1611"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B715" r:id="rId1612"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C715" r:id="rId1613"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E715" r:id="rId1614"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B716" r:id="rId1615"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C716" r:id="rId1616"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E716" r:id="rId1617"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B718" r:id="rId1618"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C718" r:id="rId1619"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E718" r:id="rId1620"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D720" r:id="rId1621"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B721" r:id="rId1622"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E721" r:id="rId1623"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B722" r:id="rId1624"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E722" r:id="rId1625"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B723" r:id="rId1626"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E723" r:id="rId1627"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B724" r:id="rId1628"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E724" r:id="rId1629"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B725" r:id="rId1630"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C725" r:id="rId1631"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E725" r:id="rId1632"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B726" r:id="rId1633"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C726" r:id="rId1634"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E726" r:id="rId1635"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C727" r:id="rId1636"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E727" r:id="rId1637"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B728" r:id="rId1638"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C728" r:id="rId1639"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E728" r:id="rId1640"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B729" r:id="rId1641"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C729" r:id="rId1642"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E729" r:id="rId1643"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C730" r:id="rId1644"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E730" r:id="rId1645"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C731" r:id="rId1646"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E731" r:id="rId1647"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B732" r:id="rId1648"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C732" r:id="rId1649"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E732" r:id="rId1650"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B733" r:id="rId1651"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E733" r:id="rId1652"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B734" r:id="rId1653"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E734" r:id="rId1654"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B735" r:id="rId1655"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E735" r:id="rId1656"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B736" r:id="rId1657"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C736" r:id="rId1658"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E736" r:id="rId1659"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B737" r:id="rId1660"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E737" r:id="rId1661"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C738" r:id="rId1662"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E738" r:id="rId1663"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C739" r:id="rId1664"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E739" r:id="rId1665"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B740" r:id="rId1666"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C740" r:id="rId1667"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E740" r:id="rId1668"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B741" r:id="rId1669"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C741" r:id="rId1670"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E741" r:id="rId1671"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C742" r:id="rId1672"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E742" r:id="rId1673"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B743" r:id="rId1674"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C743" r:id="rId1675"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E743" r:id="rId1676"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C744" r:id="rId1677"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E744" r:id="rId1678"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B745" r:id="rId1679"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E745" r:id="rId1680"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B746" r:id="rId1681"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C746" r:id="rId1682"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E746" r:id="rId1683"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B747" r:id="rId1684"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E747" r:id="rId1685"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B748" r:id="rId1686"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C748" r:id="rId1687"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E748" r:id="rId1688"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B749" r:id="rId1689"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C749" r:id="rId1690"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E749" r:id="rId1691"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>